<commit_message>
Fix payroll formulas (correct cell references) and update use-of-funds page colors to blue
</commit_message>
<xml_diff>
--- a/use-of-funds/BLU Use-of-Funds Model.xlsx
+++ b/use-of-funds/BLU Use-of-Funds Model.xlsx
@@ -2184,15 +2184,15 @@
         </is>
       </c>
       <c r="C3" s="6">
-        <f>Assumptions!C24*2* (Summary!C3/12)</f>
+        <f>Assumptions!C23*2*(Summary!C3/12)</f>
         <v/>
       </c>
       <c r="D3" s="6">
-        <f>(Assumptions!C25*2*(3/12)) + (Assumptions!C26*2*(9/12))</f>
+        <f>(Assumptions!C24*2*(3/12))+(Assumptions!C25*2*(9/12))</f>
         <v/>
       </c>
       <c r="E3" s="6">
-        <f>Assumptions!C26*2*(Summary!C5/12)</f>
+        <f>Assumptions!C25*2*(Summary!C5/12)</f>
         <v/>
       </c>
       <c r="F3" s="6">
@@ -2212,15 +2212,15 @@
         </is>
       </c>
       <c r="C4" s="6">
-        <f>(Assumptions!C21*2*(1+Assumptions!C20)) * (Summary!C3/12)</f>
+        <f>Assumptions!C20*2*(1+Assumptions!C19)*(Summary!C3/12)</f>
         <v/>
       </c>
       <c r="D4" s="6">
-        <f>(Assumptions!C21*2*(1+Assumptions!C20)) * (Summary!C4/12)</f>
+        <f>Assumptions!C20*2*(1+Assumptions!C19)*(Summary!C4/12)</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>(Assumptions!C21*2*(1+Assumptions!C20)) * (Summary!C5/12)</f>
+        <f>Assumptions!C20*2*(1+Assumptions!C19)*(Summary!C5/12)</f>
         <v/>
       </c>
       <c r="F4" s="6">
@@ -2243,11 +2243,11 @@
         <v>0</v>
       </c>
       <c r="D5" s="6">
-        <f>(Assumptions!C22*1*(1+Assumptions!C20)) * (Summary!C4/12)</f>
+        <f>Assumptions!C21*1*(1+Assumptions!C19)*(Summary!C4/12)</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>(Assumptions!C22*2*(1+Assumptions!C20)) * (Summary!C5/12)</f>
+        <f>Assumptions!C21*2*(1+Assumptions!C19)*(Summary!C5/12)</f>
         <v/>
       </c>
       <c r="F5" s="6">

</xml_diff>

<commit_message>
Fix financial model: Correct Tranche C founders pay and resolve #REF! errors
- Fixed Tranche C founders pay from  to  (corrected cell reference from Assumptions!C25 to Assumptions!C24)
- Fixed all #REF! errors by correcting row references in Total Allocation formulas
- Updated row references for S&M (C10), R&D (C12), Infra (C14), G&A (C17)
- Fixed Surplus/Deficit formulas to reference correct rows (19-20 instead of 23-24)
- Corrected all SUM formulas to reference proper data rows
- Updated references in other sheets (Timeline, Monthly_Burn) to match corrected row numbers
</commit_message>
<xml_diff>
--- a/use-of-funds/BLU Use-of-Funds Model.xlsx
+++ b/use-of-funds/BLU Use-of-Funds Model.xlsx
@@ -958,7 +958,7 @@
         </is>
       </c>
       <c r="B3" s="6">
-        <f>Assumptions!C22</f>
+        <f>Assumptions!C21</f>
         <v/>
       </c>
       <c r="C3" s="5" t="n">
@@ -2184,15 +2184,15 @@
         </is>
       </c>
       <c r="C3" s="6">
-        <f>Assumptions!C23*2*(Summary!C3/12)</f>
+        <f>Assumptions!C22*2*(Summary!C3/12)</f>
         <v/>
       </c>
       <c r="D3" s="6">
-        <f>(Assumptions!C24*2*(3/12))+(Assumptions!C25*2*(9/12))</f>
+        <f>(Assumptions!C23*2*(3/12))+(Assumptions!C24*2*(9/12))</f>
         <v/>
       </c>
       <c r="E3" s="6">
-        <f>Assumptions!C25*2*(Summary!C5/12)</f>
+        <f>Assumptions!C24*2*(Summary!C5/12)</f>
         <v/>
       </c>
       <c r="F3" s="6">
@@ -2304,7 +2304,7 @@
         <v>100000</v>
       </c>
       <c r="F7" s="6">
-        <f>SUM(C8:E8)</f>
+        <f>SUM(C7:E7)</f>
         <v/>
       </c>
     </row>
@@ -2329,7 +2329,7 @@
         <v>150000</v>
       </c>
       <c r="F8" s="6">
-        <f>SUM(C9:E9)</f>
+        <f>SUM(C8:E8)</f>
         <v/>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
         <v>60000</v>
       </c>
       <c r="F9" s="6">
-        <f>SUM(C10:E10)</f>
+        <f>SUM(C9:E9)</f>
         <v/>
       </c>
     </row>
@@ -2370,19 +2370,19 @@
         </is>
       </c>
       <c r="C10" s="6">
-        <f>SUM(C8:C10)</f>
+        <f>SUM(C7:C9)</f>
         <v/>
       </c>
       <c r="D10" s="6">
-        <f>SUM(D8:D10)</f>
+        <f>SUM(D7:D9)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>SUM(E8:E10)</f>
+        <f>SUM(E7:E9)</f>
         <v/>
       </c>
       <c r="F10" s="6">
-        <f>SUM(F8:F10)</f>
+        <f>SUM(F7:F9)</f>
         <v/>
       </c>
     </row>
@@ -2407,7 +2407,7 @@
         <v>50000</v>
       </c>
       <c r="F11" s="7">
-        <f>SUM(C13:E13)</f>
+        <f>SUM(C11:E11)</f>
         <v/>
       </c>
     </row>
@@ -2423,19 +2423,19 @@
         </is>
       </c>
       <c r="C12" s="6">
-        <f>C13</f>
+        <f>C11</f>
         <v/>
       </c>
       <c r="D12" s="6">
-        <f>D13</f>
+        <f>D11</f>
         <v/>
       </c>
       <c r="E12" s="6">
-        <f>E13</f>
+        <f>E11</f>
         <v/>
       </c>
       <c r="F12" s="6">
-        <f>F13</f>
+        <f>F11</f>
         <v/>
       </c>
     </row>
@@ -2451,7 +2451,7 @@
         </is>
       </c>
       <c r="C13" s="6">
-        <f>Infra_Estimates!F6* (Summary!C3/12)</f>
+        <f>Infra_Estimates!F6*(Summary!C3/12)</f>
         <v/>
       </c>
       <c r="D13" s="6">
@@ -2463,7 +2463,7 @@
         <v/>
       </c>
       <c r="F13" s="6">
-        <f>SUM(C16:E16)</f>
+        <f>SUM(C13:E13)</f>
         <v/>
       </c>
     </row>
@@ -2479,19 +2479,19 @@
         </is>
       </c>
       <c r="C14" s="7">
-        <f>C16</f>
+        <f>C13</f>
         <v/>
       </c>
       <c r="D14" s="7">
-        <f>D16</f>
+        <f>D13</f>
         <v/>
       </c>
       <c r="E14" s="7">
-        <f>E16</f>
+        <f>E13</f>
         <v/>
       </c>
       <c r="F14" s="7">
-        <f>F16</f>
+        <f>F13</f>
         <v/>
       </c>
     </row>
@@ -2516,7 +2516,7 @@
         <v>40000</v>
       </c>
       <c r="F15" s="6">
-        <f>SUM(C19:E19)</f>
+        <f>SUM(C15:E15)</f>
         <v/>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
         <v>30000</v>
       </c>
       <c r="F16" s="6">
-        <f>SUM(C20:E20)</f>
+        <f>SUM(C16:E16)</f>
         <v/>
       </c>
     </row>
@@ -2557,19 +2557,19 @@
         </is>
       </c>
       <c r="C17" s="7">
-        <f>SUM(C19:C20)</f>
+        <f>SUM(C15:C16)</f>
         <v/>
       </c>
       <c r="D17" s="7">
-        <f>SUM(D19:D20)</f>
+        <f>SUM(D15:D16)</f>
         <v/>
       </c>
       <c r="E17" s="7">
-        <f>SUM(E19:E20)</f>
+        <f>SUM(E15:E16)</f>
         <v/>
       </c>
       <c r="F17" s="7">
-        <f>SUM(F19:F20)</f>
+        <f>SUM(F15:F16)</f>
         <v/>
       </c>
     </row>
@@ -2589,19 +2589,19 @@
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" s="6">
-        <f>SUM(C6,C11,C14,C17,C21)</f>
+        <f>SUM(C6,C10,C12,C14,C17)</f>
         <v/>
       </c>
       <c r="D19" s="6">
-        <f>SUM(D6,D11,D14,D17,D21)</f>
+        <f>SUM(D6,D10,D12,D14,D17)</f>
         <v/>
       </c>
       <c r="E19" s="6">
-        <f>SUM(E6,E11,E14,E17,E21)</f>
+        <f>SUM(E6,E10,E12,E14,E17)</f>
         <v/>
       </c>
       <c r="F19" s="6">
-        <f>SUM(F6,F11,F14,F17,F21)</f>
+        <f>SUM(F6,F10,F12,F14,F17)</f>
         <v/>
       </c>
     </row>
@@ -2625,7 +2625,7 @@
         <v/>
       </c>
       <c r="F20" s="6">
-        <f>SUM(C24:E24)</f>
+        <f>SUM(C20:E20)</f>
         <v/>
       </c>
     </row>
@@ -2637,19 +2637,19 @@
       </c>
       <c r="B21" s="3" t="inlineStr"/>
       <c r="C21" s="7">
-        <f>C24-C23</f>
+        <f>C20-C19</f>
         <v/>
       </c>
       <c r="D21" s="7">
-        <f>D24-D23</f>
+        <f>D20-D19</f>
         <v/>
       </c>
       <c r="E21" s="7">
-        <f>E24-E23</f>
+        <f>E20-E19</f>
         <v/>
       </c>
       <c r="F21" s="7">
-        <f>F24-F23</f>
+        <f>F20-F19</f>
         <v/>
       </c>
     </row>
@@ -3546,19 +3546,19 @@
         <v/>
       </c>
       <c r="G3" s="6">
-        <f>(Tranche_Detail!C11) / Summary!C3</f>
+        <f>(Tranche_Detail!C10) / Summary!C3</f>
         <v/>
       </c>
       <c r="H3" s="6">
+        <f>(Tranche_Detail!C12) / Summary!C3</f>
+        <v/>
+      </c>
+      <c r="I3" s="6">
         <f>(Tranche_Detail!C14) / Summary!C3</f>
         <v/>
       </c>
-      <c r="I3" s="6">
+      <c r="J3" s="6">
         <f>(Tranche_Detail!C17) / Summary!C3</f>
-        <v/>
-      </c>
-      <c r="J3" s="6">
-        <f>(Tranche_Detail!C21) / Summary!C3</f>
         <v/>
       </c>
       <c r="K3" s="6">
@@ -3583,7 +3583,7 @@
         </is>
       </c>
       <c r="P3">
-        <f>(Tranche_Detail!C23) / Summary!C3</f>
+        <f>(Tranche_Detail!C19) / Summary!C3</f>
         <v/>
       </c>
     </row>
@@ -3611,19 +3611,19 @@
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(A4&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A4&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A4&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A4&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H4" s="6">
+        <f>IF(A4&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A4&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I4" s="6">
         <f>IF(A4&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A4&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I4" s="6">
+      <c r="J4" s="6">
         <f>IF(A4&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A4&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J4" s="6">
-        <f>IF(A4&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A4&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K4" s="6">
@@ -3648,7 +3648,7 @@
         </is>
       </c>
       <c r="P4">
-        <f>(Tranche_Detail!D23) / Summary!C4</f>
+        <f>(Tranche_Detail!D19) / Summary!C4</f>
         <v/>
       </c>
     </row>
@@ -3676,19 +3676,19 @@
         <v/>
       </c>
       <c r="G5" s="6">
-        <f>IF(A5&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A5&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A5&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A5&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H5" s="6">
+        <f>IF(A5&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A5&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I5" s="6">
         <f>IF(A5&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A5&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I5" s="6">
+      <c r="J5" s="6">
         <f>IF(A5&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A5&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J5" s="6">
-        <f>IF(A5&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A5&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K5" s="6">
@@ -3713,7 +3713,7 @@
         </is>
       </c>
       <c r="P5">
-        <f>(Tranche_Detail!E23) / Summary!C5</f>
+        <f>(Tranche_Detail!E19) / Summary!C5</f>
         <v/>
       </c>
     </row>
@@ -3741,19 +3741,19 @@
         <v/>
       </c>
       <c r="G6" s="6">
-        <f>IF(A6&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A6&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A6&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A6&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H6" s="6">
+        <f>IF(A6&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A6&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I6" s="6">
         <f>IF(A6&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A6&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I6" s="6">
+      <c r="J6" s="6">
         <f>IF(A6&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A6&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J6" s="6">
-        <f>IF(A6&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A6&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K6" s="6">
@@ -3797,19 +3797,19 @@
         <v/>
       </c>
       <c r="G7" s="6">
-        <f>IF(A7&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A7&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A7&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A7&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H7" s="6">
+        <f>IF(A7&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A7&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I7" s="6">
         <f>IF(A7&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A7&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I7" s="6">
+      <c r="J7" s="6">
         <f>IF(A7&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A7&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J7" s="6">
-        <f>IF(A7&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A7&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K7" s="6">
@@ -3862,19 +3862,19 @@
         <v/>
       </c>
       <c r="G8" s="6">
-        <f>IF(A8&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A8&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A8&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A8&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H8" s="6">
+        <f>IF(A8&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A8&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I8" s="6">
         <f>IF(A8&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A8&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I8" s="6">
+      <c r="J8" s="6">
         <f>IF(A8&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A8&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J8" s="6">
-        <f>IF(A8&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A8&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K8" s="6">
@@ -3899,7 +3899,7 @@
         </is>
       </c>
       <c r="P8">
-        <f>(Tranche_Detail!C11) / Summary!C3</f>
+        <f>(Tranche_Detail!C10) / Summary!C3</f>
         <v/>
       </c>
     </row>
@@ -3927,19 +3927,19 @@
         <v/>
       </c>
       <c r="G9" s="6">
-        <f>IF(A9&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A9&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A9&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A9&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H9" s="6">
+        <f>IF(A9&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A9&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I9" s="6">
         <f>IF(A9&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A9&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I9" s="6">
+      <c r="J9" s="6">
         <f>IF(A9&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A9&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J9" s="6">
-        <f>IF(A9&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A9&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K9" s="6">
@@ -3983,19 +3983,19 @@
         <v/>
       </c>
       <c r="G10" s="6">
-        <f>IF(A10&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A10&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A10&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A10&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H10" s="6">
+        <f>IF(A10&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A10&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I10" s="6">
         <f>IF(A10&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A10&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I10" s="6">
+      <c r="J10" s="6">
         <f>IF(A10&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A10&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J10" s="6">
-        <f>IF(A10&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A10&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K10" s="6">
@@ -4039,19 +4039,19 @@
         <v/>
       </c>
       <c r="G11" s="6">
-        <f>IF(A11&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A11&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A11&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A11&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H11" s="6">
+        <f>IF(A11&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A11&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I11" s="6">
         <f>IF(A11&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A11&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I11" s="6">
+      <c r="J11" s="6">
         <f>IF(A11&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A11&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J11" s="6">
-        <f>IF(A11&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A11&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K11" s="6">
@@ -4096,19 +4096,19 @@
         <v/>
       </c>
       <c r="G12" s="6">
-        <f>IF(A12&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A12&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A12&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A12&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H12" s="6">
+        <f>IF(A12&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A12&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I12" s="6">
         <f>IF(A12&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A12&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I12" s="6">
+      <c r="J12" s="6">
         <f>IF(A12&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A12&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J12" s="6">
-        <f>IF(A12&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A12&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K12" s="6">
@@ -4152,19 +4152,19 @@
         <v/>
       </c>
       <c r="G13" s="6">
-        <f>IF(A13&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A13&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A13&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A13&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H13" s="6">
+        <f>IF(A13&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A13&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I13" s="6">
         <f>IF(A13&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A13&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I13" s="6">
+      <c r="J13" s="6">
         <f>IF(A13&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A13&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J13" s="6">
-        <f>IF(A13&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A13&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K13" s="6">
@@ -4208,19 +4208,19 @@
         <v/>
       </c>
       <c r="G14" s="6">
-        <f>IF(A14&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A14&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A14&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A14&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H14" s="6">
+        <f>IF(A14&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A14&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I14" s="6">
         <f>IF(A14&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A14&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I14" s="6">
+      <c r="J14" s="6">
         <f>IF(A14&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A14&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J14" s="6">
-        <f>IF(A14&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A14&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K14" s="6">
@@ -4264,19 +4264,19 @@
         <v/>
       </c>
       <c r="G15" s="6">
-        <f>IF(A15&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A15&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A15&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A15&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H15" s="6">
+        <f>IF(A15&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A15&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I15" s="6">
         <f>IF(A15&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A15&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I15" s="6">
+      <c r="J15" s="6">
         <f>IF(A15&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A15&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J15" s="6">
-        <f>IF(A15&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A15&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K15" s="6">
@@ -4320,19 +4320,19 @@
         <v/>
       </c>
       <c r="G16" s="6">
-        <f>IF(A16&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A16&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A16&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A16&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H16" s="6">
+        <f>IF(A16&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A16&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I16" s="6">
         <f>IF(A16&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A16&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I16" s="6">
+      <c r="J16" s="6">
         <f>IF(A16&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A16&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J16" s="6">
-        <f>IF(A16&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A16&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K16" s="6">
@@ -4376,19 +4376,19 @@
         <v/>
       </c>
       <c r="G17" s="6">
-        <f>IF(A17&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A17&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A17&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A17&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H17" s="6">
+        <f>IF(A17&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A17&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I17" s="6">
         <f>IF(A17&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A17&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I17" s="6">
+      <c r="J17" s="6">
         <f>IF(A17&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A17&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J17" s="6">
-        <f>IF(A17&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A17&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K17" s="6">
@@ -4432,19 +4432,19 @@
         <v/>
       </c>
       <c r="G18" s="6">
-        <f>IF(A18&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A18&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A18&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A18&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H18" s="6">
+        <f>IF(A18&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A18&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I18" s="6">
         <f>IF(A18&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A18&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I18" s="6">
+      <c r="J18" s="6">
         <f>IF(A18&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A18&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J18" s="6">
-        <f>IF(A18&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A18&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K18" s="6">
@@ -4488,19 +4488,19 @@
         <v/>
       </c>
       <c r="G19" s="6">
-        <f>IF(A19&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A19&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A19&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A19&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H19" s="6">
+        <f>IF(A19&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A19&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I19" s="6">
         <f>IF(A19&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A19&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I19" s="6">
+      <c r="J19" s="6">
         <f>IF(A19&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A19&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J19" s="6">
-        <f>IF(A19&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A19&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K19" s="6">
@@ -4544,19 +4544,19 @@
         <v/>
       </c>
       <c r="G20" s="6">
-        <f>IF(A20&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A20&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A20&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A20&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H20" s="6">
+        <f>IF(A20&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A20&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I20" s="6">
         <f>IF(A20&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A20&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I20" s="6">
+      <c r="J20" s="6">
         <f>IF(A20&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A20&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J20" s="6">
-        <f>IF(A20&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A20&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K20" s="6">
@@ -4600,19 +4600,19 @@
         <v/>
       </c>
       <c r="G21" s="6">
-        <f>IF(A21&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A21&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A21&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A21&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H21" s="6">
+        <f>IF(A21&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A21&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I21" s="6">
         <f>IF(A21&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A21&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I21" s="6">
+      <c r="J21" s="6">
         <f>IF(A21&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A21&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J21" s="6">
-        <f>IF(A21&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A21&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K21" s="6">
@@ -4656,19 +4656,19 @@
         <v/>
       </c>
       <c r="G22" s="6">
-        <f>IF(A22&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A22&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A22&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A22&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H22" s="6">
+        <f>IF(A22&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A22&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I22" s="6">
         <f>IF(A22&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A22&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I22" s="6">
+      <c r="J22" s="6">
         <f>IF(A22&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A22&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J22" s="6">
-        <f>IF(A22&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A22&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K22" s="6">
@@ -4712,19 +4712,19 @@
         <v/>
       </c>
       <c r="G23" s="6">
-        <f>IF(A23&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A23&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A23&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A23&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H23" s="6">
+        <f>IF(A23&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A23&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I23" s="6">
         <f>IF(A23&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A23&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I23" s="6">
+      <c r="J23" s="6">
         <f>IF(A23&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A23&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J23" s="6">
-        <f>IF(A23&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A23&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K23" s="6">
@@ -4769,19 +4769,19 @@
         <v/>
       </c>
       <c r="G24" s="6">
-        <f>IF(A24&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A24&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A24&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A24&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H24" s="6">
+        <f>IF(A24&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A24&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I24" s="6">
         <f>IF(A24&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A24&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I24" s="6">
+      <c r="J24" s="6">
         <f>IF(A24&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A24&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J24" s="6">
-        <f>IF(A24&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A24&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K24" s="6">
@@ -4825,19 +4825,19 @@
         <v/>
       </c>
       <c r="G25" s="6">
-        <f>IF(A25&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A25&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A25&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A25&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H25" s="6">
+        <f>IF(A25&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A25&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I25" s="6">
         <f>IF(A25&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A25&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I25" s="6">
+      <c r="J25" s="6">
         <f>IF(A25&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A25&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J25" s="6">
-        <f>IF(A25&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A25&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K25" s="6">
@@ -4881,19 +4881,19 @@
         <v/>
       </c>
       <c r="G26" s="6">
-        <f>IF(A26&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A26&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A26&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A26&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H26" s="6">
+        <f>IF(A26&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A26&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I26" s="6">
         <f>IF(A26&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A26&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I26" s="6">
+      <c r="J26" s="6">
         <f>IF(A26&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A26&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J26" s="6">
-        <f>IF(A26&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A26&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K26" s="6">
@@ -4937,19 +4937,19 @@
         <v/>
       </c>
       <c r="G27" s="6">
-        <f>IF(A27&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A27&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A27&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A27&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H27" s="6">
+        <f>IF(A27&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A27&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I27" s="6">
         <f>IF(A27&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A27&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I27" s="6">
+      <c r="J27" s="6">
         <f>IF(A27&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A27&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J27" s="6">
-        <f>IF(A27&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A27&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K27" s="6">
@@ -4993,19 +4993,19 @@
         <v/>
       </c>
       <c r="G28" s="6">
-        <f>IF(A28&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A28&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A28&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A28&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H28" s="6">
+        <f>IF(A28&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A28&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I28" s="6">
         <f>IF(A28&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A28&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I28" s="6">
+      <c r="J28" s="6">
         <f>IF(A28&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A28&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J28" s="6">
-        <f>IF(A28&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A28&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K28" s="6">
@@ -5049,19 +5049,19 @@
         <v/>
       </c>
       <c r="G29" s="6">
-        <f>IF(A29&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A29&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A29&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A29&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H29" s="6">
+        <f>IF(A29&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A29&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I29" s="6">
         <f>IF(A29&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A29&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I29" s="6">
+      <c r="J29" s="6">
         <f>IF(A29&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A29&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J29" s="6">
-        <f>IF(A29&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A29&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K29" s="6">
@@ -5105,19 +5105,19 @@
         <v/>
       </c>
       <c r="G30" s="6">
-        <f>IF(A30&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A30&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A30&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A30&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H30" s="6">
+        <f>IF(A30&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A30&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I30" s="6">
         <f>IF(A30&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A30&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I30" s="6">
+      <c r="J30" s="6">
         <f>IF(A30&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A30&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J30" s="6">
-        <f>IF(A30&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A30&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K30" s="6">
@@ -5161,19 +5161,19 @@
         <v/>
       </c>
       <c r="G31" s="6">
-        <f>IF(A31&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A31&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A31&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A31&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H31" s="6">
+        <f>IF(A31&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A31&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I31" s="6">
         <f>IF(A31&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A31&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I31" s="6">
+      <c r="J31" s="6">
         <f>IF(A31&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A31&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J31" s="6">
-        <f>IF(A31&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A31&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K31" s="6">
@@ -5217,19 +5217,19 @@
         <v/>
       </c>
       <c r="G32" s="6">
-        <f>IF(A32&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A32&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A32&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A32&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H32" s="6">
+        <f>IF(A32&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A32&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I32" s="6">
         <f>IF(A32&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A32&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I32" s="6">
+      <c r="J32" s="6">
         <f>IF(A32&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A32&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J32" s="6">
-        <f>IF(A32&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A32&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K32" s="6">
@@ -5273,19 +5273,19 @@
         <v/>
       </c>
       <c r="G33" s="6">
-        <f>IF(A33&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A33&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A33&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A33&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H33" s="6">
+        <f>IF(A33&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A33&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I33" s="6">
         <f>IF(A33&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A33&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I33" s="6">
+      <c r="J33" s="6">
         <f>IF(A33&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A33&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J33" s="6">
-        <f>IF(A33&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A33&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K33" s="6">
@@ -5329,19 +5329,19 @@
         <v/>
       </c>
       <c r="G34" s="6">
-        <f>IF(A34&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A34&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A34&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A34&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H34" s="6">
+        <f>IF(A34&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A34&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I34" s="6">
         <f>IF(A34&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A34&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I34" s="6">
+      <c r="J34" s="6">
         <f>IF(A34&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A34&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J34" s="6">
-        <f>IF(A34&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A34&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K34" s="6">
@@ -5385,19 +5385,19 @@
         <v/>
       </c>
       <c r="G35" s="6">
-        <f>IF(A35&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A35&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A35&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A35&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H35" s="6">
+        <f>IF(A35&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A35&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I35" s="6">
         <f>IF(A35&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A35&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I35" s="6">
+      <c r="J35" s="6">
         <f>IF(A35&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A35&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J35" s="6">
-        <f>IF(A35&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A35&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K35" s="6">
@@ -5441,19 +5441,19 @@
         <v/>
       </c>
       <c r="G36" s="6">
-        <f>IF(A36&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A36&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A36&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A36&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H36" s="6">
+        <f>IF(A36&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A36&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I36" s="6">
         <f>IF(A36&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A36&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I36" s="6">
+      <c r="J36" s="6">
         <f>IF(A36&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A36&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J36" s="6">
-        <f>IF(A36&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A36&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K36" s="6">
@@ -5497,19 +5497,19 @@
         <v/>
       </c>
       <c r="G37" s="6">
-        <f>IF(A37&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A37&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A37&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A37&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H37" s="6">
+        <f>IF(A37&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A37&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I37" s="6">
         <f>IF(A37&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A37&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I37" s="6">
+      <c r="J37" s="6">
         <f>IF(A37&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A37&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J37" s="6">
-        <f>IF(A37&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A37&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K37" s="6">
@@ -5553,19 +5553,19 @@
         <v/>
       </c>
       <c r="G38" s="6">
-        <f>IF(A38&lt;=Summary!C3, (Tranche_Detail!C11)/Summary!C3, IF(A38&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D11)/Summary!C4, (Tranche_Detail!E11)/Summary!C5))</f>
+        <f>IF(A38&lt;=Summary!C3, (Tranche_Detail!C10)/Summary!C3, IF(A38&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D10)/Summary!C4, (Tranche_Detail!E10)/Summary!C5))</f>
         <v/>
       </c>
       <c r="H38" s="6">
+        <f>IF(A38&lt;=Summary!C3, (Tranche_Detail!C12)/Summary!C3, IF(A38&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D12)/Summary!C4, (Tranche_Detail!E12)/Summary!C5))</f>
+        <v/>
+      </c>
+      <c r="I38" s="6">
         <f>IF(A38&lt;=Summary!C3, (Tranche_Detail!C14)/Summary!C3, IF(A38&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D14)/Summary!C4, (Tranche_Detail!E14)/Summary!C5))</f>
         <v/>
       </c>
-      <c r="I38" s="6">
+      <c r="J38" s="6">
         <f>IF(A38&lt;=Summary!C3, (Tranche_Detail!C17)/Summary!C3, IF(A38&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D17)/Summary!C4, (Tranche_Detail!E17)/Summary!C5))</f>
-        <v/>
-      </c>
-      <c r="J38" s="6">
-        <f>IF(A38&lt;=Summary!C3, (Tranche_Detail!C21)/Summary!C3, IF(A38&lt;=(Summary!C3+Summary!C4), (Tranche_Detail!D21)/Summary!C4, (Tranche_Detail!E21)/Summary!C5))</f>
         <v/>
       </c>
       <c r="K38" s="6">
@@ -5645,7 +5645,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="6">
-        <f>Assumptions!C24</f>
+        <f>Assumptions!C22</f>
         <v/>
       </c>
       <c r="C3" s="6" t="n">
@@ -5667,11 +5667,11 @@
         <v>2</v>
       </c>
       <c r="B4" s="6">
+        <f>Assumptions!C23</f>
+        <v/>
+      </c>
+      <c r="C4" s="6">
         <f>Assumptions!C25</f>
-        <v/>
-      </c>
-      <c r="C4" s="6">
-        <f>Assumptions!C27</f>
         <v/>
       </c>
       <c r="D4" t="inlineStr">
@@ -5690,11 +5690,11 @@
         <v>3</v>
       </c>
       <c r="B5" s="6">
+        <f>Assumptions!C24</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
         <f>Assumptions!C26</f>
-        <v/>
-      </c>
-      <c r="C5" s="6">
-        <f>Assumptions!C28</f>
         <v/>
       </c>
       <c r="D5" t="inlineStr">

</xml_diff>

<commit_message>
Optimize use of funds to align with  raise
- Phase in Stage 3 founder pay: First 6 months at Stage 2, last 6 months at Stage 3 (saves ~)
- Delay engineer hiring: Reduce Tranche C by 3 months (saves ~)
- Delay sales hiring: Phase in second sales hire 3 months later (saves ~)
- Reduce S&M spend: Lower Tranche C Ambassador and Social/Digital CAC (saves ~)
- Optimize R&D: Reduce Tranche C from  to  (saves )
- Optimize G&A: Reduce Office & Misc from  to  (saves )
- Total estimated savings: ~, bringing overage from ~ to ~

These changes align capital allocation with revenue milestones, preserve capital efficiency, and maintain realistic growth projections while staying within the  raise structure.
</commit_message>
<xml_diff>
--- a/use-of-funds/BLU Use-of-Funds Model.xlsx
+++ b/use-of-funds/BLU Use-of-Funds Model.xlsx
@@ -2192,7 +2192,7 @@
         <v/>
       </c>
       <c r="E3" s="6">
-        <f>Assumptions!C24*2*(Summary!C5/12)</f>
+        <f>(Assumptions!C23*2*(6/12))+(Assumptions!C24*2*(6/12))</f>
         <v/>
       </c>
       <c r="F3" s="6">
@@ -2220,7 +2220,7 @@
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>Assumptions!C20*2*(1+Assumptions!C19)*(Summary!C5/12)</f>
+        <f>Assumptions!C20*2*(1+Assumptions!C19)*((Summary!C5-3)/12)</f>
         <v/>
       </c>
       <c r="F4" s="6">
@@ -2247,7 +2247,7 @@
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>Assumptions!C21*2*(1+Assumptions!C19)*(Summary!C5/12)</f>
+        <f>Assumptions!C21*1*(1+Assumptions!C19)*((Summary!C5-3)/12)+Assumptions!C21*2*(1+Assumptions!C19)*(3/12)</f>
         <v/>
       </c>
       <c r="F5" s="6">
@@ -2301,7 +2301,7 @@
         <v>50000</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="F7" s="6">
         <f>SUM(C7:E7)</f>
@@ -2326,7 +2326,7 @@
         <v>75000</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="F8" s="6">
         <f>SUM(C8:E8)</f>
@@ -2404,7 +2404,7 @@
         <v>30000</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>50000</v>
+        <v>40000</v>
       </c>
       <c r="F11" s="7">
         <f>SUM(C11:E11)</f>
@@ -2538,7 +2538,7 @@
         <v>20000</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>30000</v>
+        <v>20000</v>
       </c>
       <c r="F16" s="6">
         <f>SUM(C16:E16)</f>

</xml_diff>

<commit_message>
Fix salary progression: Founder pay now scales UP over time, tied to milestones
- Tranche A: Stage 1 (.5k/month per founder) - current pay
- Tranche B: Phases from Stage 1 to Stage 2 (/month) when  MRR milestone hit
- Tranche C: Maintains Stage 2 (/month) - conservative approach, prioritizing Engineers and growth
- Removed salary decreases - all salaries now scale UP or stay constant
- Engineer salaries scale UP (9 months â†’ 12 months â†’ 12 months)
- Founder pay tied to performance milestones, not just tranche receipt
- Web page updated to reflect performance-based compensation philosophy
</commit_message>
<xml_diff>
--- a/use-of-funds/BLU Use-of-Funds Model.xlsx
+++ b/use-of-funds/BLU Use-of-Funds Model.xlsx
@@ -2188,11 +2188,11 @@
         <v/>
       </c>
       <c r="D3" s="6">
-        <f>(Assumptions!C23*2*(3/12))+(Assumptions!C24*2*(9/12))</f>
+        <f>(Assumptions!C22*2*(6/12))+(Assumptions!C23*2*(6/12))</f>
         <v/>
       </c>
       <c r="E3" s="6">
-        <f>(Assumptions!C23*2*(6/12))+(Assumptions!C24*2*(6/12))</f>
+        <f>Assumptions!C23*2*(Summary!C5/12)</f>
         <v/>
       </c>
       <c r="F3" s="6">
@@ -2220,7 +2220,7 @@
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>Assumptions!C20*2*(1+Assumptions!C19)*((Summary!C5-3)/12)</f>
+        <f>Assumptions!C20*2*(1+Assumptions!C19)*(Summary!C5/12)</f>
         <v/>
       </c>
       <c r="F4" s="6">

</xml_diff>

<commit_message>
Update revenue milestones to more realistic GTM trajectory
- Tranche A: Added \-5k MRR milestone (early revenue validation)
- Tranche B: Increased from \ to \ MRR (more realistic post-PMF growth)
- Tranche C: Kept at \ MRR (now 3x from \ instead of 6.7x from \)
- Updated all web page references and spreadsheet formulas
- More defensible growth curve: 8-10x (Aâ†’B), then 3x (Bâ†’C)
- Shows confidence AND realism - early validation signals strong GTM execution
</commit_message>
<xml_diff>
--- a/use-of-funds/BLU Use-of-Funds Model.xlsx
+++ b/use-of-funds/BLU Use-of-Funds Model.xlsx
@@ -2066,7 +2066,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Tranche A Milestones Met (5 Leagues, 100 Umpires)</t>
+          <t>Tranche A Milestones Met (5 Leagues, 100 Umpires, $3-5k MRR)</t>
         </is>
       </c>
     </row>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Tranche B Milestones Met ($15k MRR, 2% Conversion)</t>
+          <t>Tranche B Milestones Met ($35k MRR, 2% Conversion)</t>
         </is>
       </c>
     </row>
@@ -5762,7 +5762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5897,24 +5897,24 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tranche A Milestones Met</t>
+          <t>Generate $3-5k MRR</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>MRR</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>4000</v>
       </c>
       <c r="E6">
-        <f>IF(F5="Met",1,0)</f>
+        <f>County_League_Model!D22</f>
         <v/>
       </c>
       <c r="F6">
@@ -5930,19 +5930,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Achieve $15k MRR</t>
+          <t>Tranche A Milestones Met</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MRR</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="E7" s="6">
-        <f>County_League_Model!D22</f>
+        <f>IF(AND(F5="Met",F6="Met"),1,0)</f>
         <v/>
       </c>
       <c r="F7">
@@ -5953,29 +5953,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Parent Conversion</t>
+          <t>Generate $3-5k MRR</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D8" s="5">
-        <f>Assumptions!C8</f>
-        <v/>
+          <t>MRR</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>4000</v>
       </c>
       <c r="E8" s="5">
-        <f>Assumptions!C8</f>
+        <f>County_League_Model!D22</f>
         <v/>
       </c>
       <c r="F8">
-        <f>IF(E8&gt;=D8,"Met","Pending")</f>
+        <f>IF(E5&gt;=D5,"Met","Pending")</f>
         <v/>
       </c>
     </row>
@@ -5987,80 +5986,81 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Coach Conversion</t>
+          <t>Achieve $35k MRR</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D9" s="5">
-        <f>Assumptions!C9</f>
-        <v/>
+          <t>MRR</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>35000</v>
       </c>
       <c r="E9" s="5">
-        <f>Assumptions!C9</f>
+        <f>County_League_Model!D22</f>
         <v/>
       </c>
       <c r="F9">
-        <f>IF(E9&gt;=D9,"Met","Pending")</f>
+        <f>IF(E7&gt;=D7,"Met","Pending")</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tranche B Milestones Met</t>
+          <t>Parent Conversion</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>1</v>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D10">
+        <f>Assumptions!C8</f>
+        <v/>
       </c>
       <c r="E10">
-        <f>IF(AND(F7="Met",F8="Met",F9="Met"),1,0)</f>
+        <f>Assumptions!C8</f>
         <v/>
       </c>
       <c r="F10">
-        <f>IF(E10&gt;=D10,"Met","Pending")</f>
+        <f>IF(E9&gt;=D9,"Met","Pending")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Achieve $100k MRR</t>
+          <t>Coach Conversion</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MRR</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>100000</v>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D11" s="6">
+        <f>Assumptions!C9</f>
+        <v/>
       </c>
       <c r="E11" s="6">
-        <f>County_League_Model!D22</f>
+        <f>Assumptions!C9</f>
         <v/>
       </c>
       <c r="F11">
-        <f>IF(E11&gt;=D11,"Met","Pending")</f>
+        <f>IF(E10&gt;=D10,"Met","Pending")</f>
         <v/>
       </c>
     </row>
@@ -6072,23 +6072,79 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>Tranche B Milestones Met</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <f>IF(AND(F8="Met",F9="Met",F10="Met"),1,0)</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f>IF(E11&gt;=D11,"Met","Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Achieve $100k MRR</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MRR</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E13">
+        <f>County_League_Model!D22</f>
+        <v/>
+      </c>
+      <c r="F13">
+        <f>IF(E12&gt;=D12,"Met","Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>Org Contracts</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D14" t="n">
         <v>10</v>
       </c>
-      <c r="E12">
+      <c r="E14">
         <f>County_League_Model!D15</f>
         <v/>
       </c>
-      <c r="F12">
-        <f>IF(E12&gt;=D12,"Met","Pending")</f>
+      <c r="F14">
+        <f>IF(E13&gt;=D13,"Met","Pending")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix duplicate milestone entry in spreadsheet
</commit_message>
<xml_diff>
--- a/use-of-funds/BLU Use-of-Funds Model.xlsx
+++ b/use-of-funds/BLU Use-of-Funds Model.xlsx
@@ -5762,7 +5762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5953,12 +5953,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Generate $3-5k MRR</t>
+          <t>Achieve $35k MRR</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -5967,14 +5967,14 @@
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>4000</v>
+        <v>35000</v>
       </c>
       <c r="E8" s="5">
         <f>County_League_Model!D22</f>
         <v/>
       </c>
       <c r="F8">
-        <f>IF(E5&gt;=D5,"Met","Pending")</f>
+        <f>IF(E8&gt;=D8,"Met","Pending")</f>
         <v/>
       </c>
     </row>
@@ -5986,23 +5986,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Achieve $35k MRR</t>
+          <t>Parent Conversion</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MRR</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>35000</v>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D9" s="5">
+        <f>Assumptions!C8</f>
+        <v/>
       </c>
       <c r="E9" s="5">
-        <f>County_League_Model!D22</f>
+        <f>Assumptions!C8</f>
         <v/>
       </c>
       <c r="F9">
-        <f>IF(E7&gt;=D7,"Met","Pending")</f>
+        <f>IF(E9&gt;=D9,"Met","Pending")</f>
         <v/>
       </c>
     </row>
@@ -6014,7 +6015,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Parent Conversion</t>
+          <t>Coach Conversion</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -6023,44 +6024,43 @@
         </is>
       </c>
       <c r="D10">
-        <f>Assumptions!C8</f>
+        <f>Assumptions!C9</f>
         <v/>
       </c>
       <c r="E10">
-        <f>Assumptions!C8</f>
+        <f>Assumptions!C9</f>
         <v/>
       </c>
       <c r="F10">
-        <f>IF(E9&gt;=D9,"Met","Pending")</f>
+        <f>IF(E10&gt;=D10,"Met","Pending")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Coach Conversion</t>
+          <t>Tranche B Milestones Met</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D11" s="6">
-        <f>Assumptions!C9</f>
-        <v/>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="E11" s="6">
-        <f>Assumptions!C9</f>
+        <f>IF(AND(F8="Met",F9="Met",F10="Met"),1,0)</f>
         <v/>
       </c>
       <c r="F11">
-        <f>IF(E10&gt;=D10,"Met","Pending")</f>
+        <f>IF(E11&gt;=D11,"Met","Pending")</f>
         <v/>
       </c>
     </row>
@@ -6072,23 +6072,23 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Tranche B Milestones Met</t>
+          <t>Achieve $100k MRR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>MRR</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>100000</v>
       </c>
       <c r="E12">
-        <f>IF(AND(F8="Met",F9="Met",F10="Met"),1,0)</f>
+        <f>County_League_Model!D22</f>
         <v/>
       </c>
       <c r="F12">
-        <f>IF(E11&gt;=D11,"Met","Pending")</f>
+        <f>IF(E12&gt;=D12,"Met","Pending")</f>
         <v/>
       </c>
     </row>
@@ -6100,50 +6100,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Achieve $100k MRR</t>
+          <t>Org Contracts</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MRR</t>
+          <t>Count</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>100000</v>
+        <v>10</v>
       </c>
       <c r="E13">
-        <f>County_League_Model!D22</f>
+        <f>County_League_Model!D15</f>
         <v/>
       </c>
       <c r="F13">
-        <f>IF(E12&gt;=D12,"Met","Pending")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Org Contracts</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>10</v>
-      </c>
-      <c r="E14">
-        <f>County_League_Model!D15</f>
-        <v/>
-      </c>
-      <c r="F14">
         <f>IF(E13&gt;=D13,"Met","Pending")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Regenerate Excel file with B2C-only strategy: Funnel_Model engine, 3% coach conversion, zero org revenue, Growth & Partnerships team, dynamic CAC formulas
</commit_message>
<xml_diff>
--- a/use-of-funds/BLU Use-of-Funds Model.xlsx
+++ b/use-of-funds/BLU Use-of-Funds Model.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tranche_Detail" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="County_League_Model" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funnel_Model" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash_Runway" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pay_Triggers" sheetId="8" state="visible" r:id="rId8"/>
@@ -547,7 +547,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>'County_League_Model' projects user growth and ARR based on your assumptions.</t>
+          <t>Look at the 'Funnel_Model' tab. This is the engine of the entire spreadsheet. It projects a 3-year forecast starting with 'New Umpires Acquired' as the main input, calculates 'Total Freemium Users Reached' (our viral loop), and then 'Total ARR' based on our B2C conversion rates. All other tabs pull their data from this Funnel_Model.</t>
         </is>
       </c>
     </row>
@@ -825,15 +825,15 @@
         </is>
       </c>
       <c r="B3" s="6">
-        <f>(County_League_Model!D9*Scenarios!B3*Assumptions!D11) + (County_League_Model!D10*Scenarios!B4*Assumptions!D11) + (County_League_Model!D15*Scenarios!B6)</f>
+        <f>(Funnel_Model!D26*Scenarios!B3*Assumptions!D11) + (Funnel_Model!D27*Scenarios!B4*Assumptions!D11)</f>
         <v/>
       </c>
       <c r="C3" s="6">
-        <f>County_League_Model!D21</f>
+        <f>Funnel_Model!D30</f>
         <v/>
       </c>
       <c r="D3" s="6">
-        <f>(County_League_Model!D9*Scenarios!D3*Assumptions!E11) + (County_League_Model!D10*Scenarios!D4*Assumptions!E11) + (County_League_Model!D15*Scenarios!D6)</f>
+        <f>(Funnel_Model!D26*Scenarios!D3*Assumptions!E11) + (Funnel_Model!D27*Scenarios!D4*Assumptions!E11)</f>
         <v/>
       </c>
     </row>
@@ -844,15 +844,15 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>(County_League_Model!D9*Scenarios!B3) + (County_League_Model!D10*Scenarios!B4) + (County_League_Model!D15)</f>
+        <f>(Funnel_Model!D26*Scenarios!B3) + (Funnel_Model!D27*Scenarios!B4)</f>
         <v/>
       </c>
       <c r="C4" s="4">
-        <f>County_League_Model!D13 + County_League_Model!D14 + County_League_Model!D15</f>
+        <f>Funnel_Model!D26 + Funnel_Model!D27</f>
         <v/>
       </c>
       <c r="D4" s="4">
-        <f>(County_League_Model!D9*Scenarios!D3) + (County_League_Model!D10*Scenarios!D4) + (County_League_Model!D15)</f>
+        <f>(Funnel_Model!D26*Scenarios!D3) + (Funnel_Model!D27*Scenarios!D4)</f>
         <v/>
       </c>
     </row>
@@ -883,7 +883,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>( (Scenarios!B7*B4) + (Scenarios!B9*County_League_Model!D15) ) / (B3*Assumptions!D14) * 12</t>
+          <t>( (Scenarios!B7*B4) ) / (B3*Assumptions!D14) * 12</t>
         </is>
       </c>
       <c r="C6" s="9">
@@ -892,7 +892,7 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>( (Scenarios!D7*D4) + (Scenarios!D9*County_League_Model!D15) ) / (D3*Assumptions!E14) * 12</t>
+          <t>( (Scenarios!D7*D4) ) / (D3*Assumptions!E14) * 12</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="4">
-        <f>County_League_Model!C8</f>
+        <f>Funnel_Model!C16</f>
         <v/>
       </c>
       <c r="E3" s="6">
@@ -1119,7 +1119,7 @@
         <v>0.5</v>
       </c>
       <c r="D4" s="4">
-        <f>(County_League_Model!C8*20)</f>
+        <f>Funnel_Model!C17</f>
         <v/>
       </c>
       <c r="E4" s="6">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Assuming 20 games/umpire/year</t>
+          <t>Total games scored in Year 2</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1196,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>E6/County_League_Model!C21</f>
+        <f>E6/Funnel_Model!C30</f>
         <v/>
       </c>
     </row>
@@ -1428,13 +1428,13 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>0.1</v>
+        <v>0.03</v>
       </c>
       <c r="D9" s="5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E9" s="5" t="n">
         <v>0.05</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>0.15</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1450,47 +1450,47 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>League/Org Conversion % (Yr 1)</t>
+          <t>Paid User Churn Rate (Annual)</t>
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>0.05</v>
+        <v>0.33</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>0.03</v>
+        <v>0.4</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.08</v>
+        <v>0.25</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Leagues converting to B2B platform</t>
+          <t>Annual churn rate for paid users (inverse of 3yr lifetime)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Pricing</t>
+          <t>Conversion</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Coach/Parent App (Annual)</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>199</v>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>199</v>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>249</v>
+          <t>League/Org Conversion % (Yr 1)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Annual subscription</t>
+          <t>B2C-only strategy - no organization revenue</t>
         </is>
       </c>
     </row>
@@ -1502,45 +1502,49 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Organization Price (Annual Avg)</t>
+          <t>Coach/Parent App (Annual)</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>5000</v>
+        <v>199</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>3500</v>
+        <v>199</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>7500</v>
+        <v>249</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Per league, custom pricing</t>
+          <t>Annual subscription</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Unit Economics</t>
+          <t>Pricing</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>User Lifetime (Years)</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D13" s="4" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F13" t="inlineStr"/>
+          <t>Organization Price (Annual Avg)</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>B2C-only strategy - no organization revenue</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1550,23 +1554,19 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Gross Margin</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E14" s="5" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Revenue minus COGS (Infra, Support)</t>
-        </is>
-      </c>
+          <t>User Lifetime (Years)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1576,47 +1576,47 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Annual Discount Rate</t>
+          <t>Gross Margin</t>
         </is>
       </c>
       <c r="C15" s="5" t="n">
-        <v>0.1</v>
+        <v>0.55</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>0.12</v>
+        <v>0.5</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.08</v>
+        <v>0.6</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>For LTV calculation (optional)</t>
+          <t>Revenue minus COGS (Infra, Support)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAC</t>
+          <t>Unit Economics</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CAC - Ambassador ($/user)</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="D16" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="E16" s="6" t="n">
-        <v>25</v>
+          <t>Annual Discount Rate</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>0.08</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Paid user (parent/coach)</t>
+          <t>For LTV calculation (optional)</t>
         </is>
       </c>
     </row>
@@ -1628,17 +1628,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CAC - Social/Digital ($/user)</t>
+          <t>CAC - Ambassador ($/user)</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1654,47 +1654,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CAC - Organization ($/league)</t>
+          <t>CAC - Social/Digital ($/user)</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>1200</v>
+        <v>80</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>1500</v>
+        <v>100</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1000</v>
+        <v>70</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>League B2B sale</t>
+          <t>Paid user (parent/coach)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>CAC</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Employer Burden</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D19" s="5" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="E19" s="5" t="n">
-        <v>0.1</v>
+          <t>CAC - Organization ($/league)</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>% on top of base salary (taxes, benefits)</t>
+          <t>B2C-only strategy - no organization CAC</t>
         </is>
       </c>
     </row>
@@ -1706,19 +1706,23 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Engineer Salary (Avg)</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>120000</v>
-      </c>
-      <c r="D20" s="6" t="n">
-        <v>110000</v>
-      </c>
-      <c r="E20" s="6" t="n">
-        <v>130000</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
+          <t>Employer Burden</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>% on top of base salary (taxes, benefits)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1728,45 +1732,41 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sales Salary (Avg)</t>
+          <t>Engineer Salary (Avg)</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>80000</v>
+        <v>120000</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>75000</v>
+        <v>110000</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>85000</v>
+        <v>130000</v>
       </c>
       <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Pay Triggers</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Founder Pay - Stage 1 (Annual)</t>
+          <t>Sales Salary (Avg)</t>
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>90000</v>
+        <v>80000</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>90000</v>
+        <v>75000</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>90000</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Annual Salary per Founder ($7.5k/mo)</t>
-        </is>
-      </c>
+        <v>85000</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1776,21 +1776,21 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Founder Pay - Stage 2 (Annual)</t>
+          <t>Founder Pay - Stage 1 (Annual)</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>120000</v>
+        <v>90000</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>120000</v>
+        <v>90000</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>120000</v>
+        <v>90000</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Annual Salary per Founder ($10k/mo)</t>
+          <t>Annual Salary per Founder ($7.5k/mo)</t>
         </is>
       </c>
     </row>
@@ -1802,21 +1802,21 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Founder Pay - Stage 3 (Annual)</t>
+          <t>Founder Pay - Stage 2 (Annual)</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>250000</v>
+        <v>120000</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>250000</v>
+        <v>120000</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>250000</v>
+        <v>120000</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Annual Salary per Founder</t>
+          <t>Annual Salary per Founder ($10k/mo)</t>
         </is>
       </c>
     </row>
@@ -1828,21 +1828,21 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MRR Trigger - Stage 2</t>
+          <t>Founder Pay - Stage 3 (Annual)</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>10000</v>
+        <v>250000</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>10000</v>
+        <v>250000</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>10000</v>
+        <v>250000</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>MRR threshold for Stage 2 pay</t>
+          <t>Annual Salary per Founder</t>
         </is>
       </c>
     </row>
@@ -1854,47 +1854,47 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MRR Trigger - Stage 3</t>
+          <t>MRR Trigger - Stage 2</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>50000</v>
+        <v>10000</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>50000</v>
+        <v>10000</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>50000</v>
+        <v>10000</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>MRR threshold for Stage 3 pay</t>
+          <t>MRR threshold for Stage 2 pay</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Funding</t>
+          <t>Pay Triggers</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tranche A</t>
+          <t>MRR Trigger - Stage 3</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>250000</v>
+        <v>50000</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>250000</v>
+        <v>50000</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>250000</v>
+        <v>50000</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>MVP &amp; Pilot</t>
+          <t>MRR threshold for Stage 3 pay</t>
         </is>
       </c>
     </row>
@@ -1906,21 +1906,21 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Tranche B</t>
+          <t>Tranche A</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>750000</v>
+        <v>250000</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>750000</v>
+        <v>250000</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>750000</v>
+        <v>250000</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Product-Market Fit</t>
+          <t>MVP &amp; Pilot</t>
         </is>
       </c>
     </row>
@@ -1932,28 +1932,49 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>Tranche B</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>750000</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>750000</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>750000</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Product-Market Fit</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Funding</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>Tranche C</t>
         </is>
       </c>
-      <c r="C29" s="6" t="n">
+      <c r="C30" s="6" t="n">
         <v>1000000</v>
       </c>
-      <c r="D29" s="6" t="n">
+      <c r="D30" s="6" t="n">
         <v>1000000</v>
       </c>
-      <c r="E29" s="6" t="n">
+      <c r="E30" s="6" t="n">
         <v>1000000</v>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>Growth</t>
         </is>
       </c>
-    </row>
-    <row r="30">
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="C31" s="4" t="n"/>
@@ -2085,7 +2106,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Drive Scalable Growth (Organization Sales)</t>
+          <t>Scale B2C Engine</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2236,7 +2257,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sales (1 -&gt; 2)</t>
+          <t>Growth &amp; Partnerships (1 -&gt; 2)</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
@@ -2294,14 +2315,17 @@
           <t>CAC - Ambassador</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>50000</v>
+      <c r="C7" s="6">
+        <f>(Funnel_Model!B22+Funnel_Model!B23)*Assumptions!C17</f>
+        <v/>
+      </c>
+      <c r="D7" s="6">
+        <f>(Funnel_Model!C22+Funnel_Model!C23)*Assumptions!C17</f>
+        <v/>
+      </c>
+      <c r="E7" s="6">
+        <f>(Funnel_Model!D22+Funnel_Model!D23)*Assumptions!C17</f>
+        <v/>
       </c>
       <c r="F7" s="6">
         <f>SUM(C7:E7)</f>
@@ -2319,14 +2343,17 @@
           <t>CAC - Social/Digital</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
-        <v>20000</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>75000</v>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>100000</v>
+      <c r="C8" s="6">
+        <f>(Funnel_Model!B22+Funnel_Model!B23)*Assumptions!C18</f>
+        <v/>
+      </c>
+      <c r="D8" s="6">
+        <f>(Funnel_Model!C22+Funnel_Model!C23)*Assumptions!C18</f>
+        <v/>
+      </c>
+      <c r="E8" s="6">
+        <f>(Funnel_Model!D22+Funnel_Model!D23)*Assumptions!C18</f>
+        <v/>
       </c>
       <c r="F8" s="6">
         <f>SUM(C8:E8)</f>
@@ -2345,13 +2372,13 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>60000</v>
+        <v>0</v>
       </c>
       <c r="F9" s="6">
         <f>SUM(C9:E9)</f>
@@ -2694,20 +2721,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>County &amp; League Growth Model (Base Scenario)</t>
+          <t>Funnel Model - Bottom-Up Revenue Projections</t>
         </is>
       </c>
     </row>
@@ -2739,417 +2766,570 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Counties Targeted (New)</t>
-        </is>
-      </c>
-      <c r="B3" s="4">
-        <f>Assumptions!C3</f>
-        <v/>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="E3" s="4">
-        <f>SUM(B3:D3)</f>
-        <v/>
-      </c>
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>New Leagues Acquired</t>
-        </is>
-      </c>
-      <c r="B4" s="4">
-        <f>B3*Assumptions!C4</f>
-        <v/>
-      </c>
-      <c r="C4" s="4">
-        <f>C3*Assumptions!C4</f>
-        <v/>
-      </c>
-      <c r="D4" s="4">
-        <f>D3*Assumptions!C4</f>
-        <v/>
-      </c>
-      <c r="E4" s="4">
-        <f>SUM(B4:D4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Total Leagues (Cumulative)</t>
-        </is>
-      </c>
-      <c r="B5" s="4">
-        <f>B4</f>
-        <v/>
-      </c>
-      <c r="C5" s="4">
-        <f>B5+C4</f>
-        <v/>
-      </c>
-      <c r="D5" s="4">
-        <f>C5+D4</f>
-        <v/>
-      </c>
-      <c r="E5" s="4">
-        <f>D5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+          <t>INPUTS</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>User Base</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Year 1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Year 2</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Year 3</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
+      <c r="A7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Total Umpires</t>
-        </is>
-      </c>
-      <c r="B8" s="4">
-        <f>B5*Assumptions!C5</f>
-        <v/>
-      </c>
-      <c r="C8" s="4">
-        <f>C5*Assumptions!C5</f>
-        <v/>
-      </c>
-      <c r="D8" s="4">
-        <f>D5*Assumptions!C5</f>
-        <v/>
-      </c>
-      <c r="E8" s="4">
-        <f>D8</f>
-        <v/>
+          <t>New Umpires Acquired</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Target from Umpire_Funnel tab</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Total Parents (Potential)</t>
-        </is>
-      </c>
-      <c r="B9" s="4">
-        <f>B8*Assumptions!C6</f>
-        <v/>
-      </c>
-      <c r="C9" s="4">
-        <f>C8*Assumptions!C6</f>
-        <v/>
-      </c>
-      <c r="D9" s="4">
-        <f>D8*Assumptions!C6</f>
-        <v/>
-      </c>
-      <c r="E9" s="4">
-        <f>D9</f>
-        <v/>
+          <t>Umpire Churn Rate</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Annual churn rate</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Total Coaches (Potential)</t>
-        </is>
-      </c>
-      <c r="B10" s="4">
-        <f>B5*Assumptions!C7</f>
-        <v/>
-      </c>
-      <c r="C10" s="4">
-        <f>C5*Assumptions!C7</f>
-        <v/>
-      </c>
-      <c r="D10" s="4">
-        <f>D5*Assumptions!C7</f>
-        <v/>
-      </c>
-      <c r="E10" s="4">
-        <f>D10</f>
-        <v/>
+          <t>Avg. Games per Umpire per Year</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Games captured annually</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Avg. Unique Players per Game</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Players reached per game</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Paid Conversions (New)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Year 1</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Year 2</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Year 3</t>
-        </is>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Avg. Parents/Coaches per Player</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>1.5</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Parents &amp; coaches per player</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Paid Parents</t>
-        </is>
-      </c>
-      <c r="B13" s="4">
-        <f>B9*Assumptions!C8</f>
-        <v/>
-      </c>
-      <c r="C13" s="4">
-        <f>C9*Assumptions!C8</f>
-        <v/>
-      </c>
-      <c r="D13" s="4">
-        <f>D9*Assumptions!C8</f>
-        <v/>
-      </c>
-      <c r="E13" s="4">
-        <f>SUM(B13:D13)</f>
-        <v/>
-      </c>
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Paid Coaches</t>
-        </is>
-      </c>
-      <c r="B14" s="4">
-        <f>B10*Assumptions!C9</f>
-        <v/>
-      </c>
-      <c r="C14" s="4">
-        <f>C10*Assumptions!C9</f>
-        <v/>
-      </c>
-      <c r="D14" s="4">
-        <f>D10*Assumptions!C9</f>
-        <v/>
-      </c>
-      <c r="E14" s="4">
-        <f>SUM(B14:D14)</f>
-        <v/>
+          <t>CALCULATIONS</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Paid Organizations</t>
+          <t>New Umpires Acquired</t>
         </is>
       </c>
       <c r="B15" s="4">
-        <f>B4*Assumptions!C10</f>
+        <f>B8</f>
         <v/>
       </c>
       <c r="C15" s="4">
-        <f>(C4*Assumptions!C10)</f>
+        <f>C8</f>
         <v/>
       </c>
       <c r="D15" s="4">
-        <f>(D4*Assumptions!C10)</f>
+        <f>D8</f>
         <v/>
       </c>
       <c r="E15" s="4">
-        <f>SUM(B15:D15)</f>
+        <f>D14</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Umpires Retained from Prior Year</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="4">
+        <f>B14*(1-B9)</f>
+        <v/>
+      </c>
+      <c r="D16" s="4">
+        <f>C16*(1-C9)</f>
+        <v/>
+      </c>
+      <c r="E16" s="4">
+        <f>D15</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Annual Recurring Revenue (ARR)</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Year 1</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Year 2</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Year 3</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Total Active Umpires</t>
+        </is>
+      </c>
+      <c r="B17" s="4">
+        <f>B14+B15</f>
+        <v/>
+      </c>
+      <c r="C17" s="4">
+        <f>C14+C15</f>
+        <v/>
+      </c>
+      <c r="D17" s="4">
+        <f>D14+D15</f>
+        <v/>
+      </c>
+      <c r="E17" s="4">
+        <f>D16</f>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Parent App Revenue</t>
-        </is>
-      </c>
-      <c r="B18" s="6">
-        <f>B13*Assumptions!C11</f>
-        <v/>
-      </c>
-      <c r="C18" s="6">
-        <f>C13*Assumptions!C11</f>
-        <v/>
-      </c>
-      <c r="D18" s="6">
-        <f>D13*Assumptions!C11</f>
-        <v/>
-      </c>
-      <c r="E18" s="6">
-        <f>SUM(B18:D18)</f>
+          <t>Total Games Scored</t>
+        </is>
+      </c>
+      <c r="B18" s="4">
+        <f>B16*B10</f>
+        <v/>
+      </c>
+      <c r="C18" s="4">
+        <f>C16*C10</f>
+        <v/>
+      </c>
+      <c r="D18" s="4">
+        <f>D16*D10</f>
+        <v/>
+      </c>
+      <c r="E18" s="4">
+        <f>D17</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Coach App Revenue</t>
-        </is>
-      </c>
-      <c r="B19" s="6">
-        <f>B14*Assumptions!C11</f>
-        <v/>
-      </c>
-      <c r="C19" s="6">
-        <f>C14*Assumptions!C11</f>
-        <v/>
-      </c>
-      <c r="D19" s="6">
-        <f>D14*Assumptions!C11</f>
-        <v/>
-      </c>
-      <c r="E19" s="6">
-        <f>SUM(B19:D19)</f>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Total Players Reached</t>
+        </is>
+      </c>
+      <c r="B19" s="4">
+        <f>B17*B11</f>
+        <v/>
+      </c>
+      <c r="C19" s="4">
+        <f>C17*C11</f>
+        <v/>
+      </c>
+      <c r="D19" s="4">
+        <f>D17*D11</f>
+        <v/>
+      </c>
+      <c r="E19" s="4">
+        <f>D18</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Organization Revenue</t>
-        </is>
-      </c>
-      <c r="B20" s="6">
-        <f>B15*Assumptions!C12</f>
-        <v/>
-      </c>
-      <c r="C20" s="6">
-        <f>C15*Assumptions!C12</f>
-        <v/>
-      </c>
-      <c r="D20" s="6">
-        <f>D15*Assumptions!C12</f>
-        <v/>
-      </c>
-      <c r="E20" s="6">
-        <f>SUM(B20:D20)</f>
+          <t>Total Freemium Users Reached (Parents/Coaches)</t>
+        </is>
+      </c>
+      <c r="B20">
+        <f>B18*B12</f>
+        <v/>
+      </c>
+      <c r="C20">
+        <f>C18*C12</f>
+        <v/>
+      </c>
+      <c r="D20">
+        <f>D18*D12</f>
+        <v/>
+      </c>
+      <c r="E20">
+        <f>D19</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Total ARR</t>
-        </is>
-      </c>
-      <c r="B21" s="6">
-        <f>SUM(B18:B20)</f>
-        <v/>
-      </c>
-      <c r="C21" s="6">
-        <f>SUM(C18:C20)</f>
-        <v/>
-      </c>
-      <c r="D21" s="6">
-        <f>SUM(D18:D20)</f>
-        <v/>
-      </c>
-      <c r="E21" s="6">
-        <f>SUM(B21:D21)</f>
-        <v/>
-      </c>
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>New Paid Parents</t>
+        </is>
+      </c>
+      <c r="B23" s="4">
+        <f>B19*Assumptions!C8</f>
+        <v/>
+      </c>
+      <c r="C23" s="4">
+        <f>C19*Assumptions!C8</f>
+        <v/>
+      </c>
+      <c r="D23" s="4">
+        <f>D19*Assumptions!C8</f>
+        <v/>
+      </c>
+      <c r="E23" s="4">
+        <f>D22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>New Paid Coaches</t>
+        </is>
+      </c>
+      <c r="B24" s="4">
+        <f>B19*Assumptions!C9</f>
+        <v/>
+      </c>
+      <c r="C24" s="4">
+        <f>C19*Assumptions!C9</f>
+        <v/>
+      </c>
+      <c r="D24" s="4">
+        <f>D19*Assumptions!C9</f>
+        <v/>
+      </c>
+      <c r="E24" s="4">
+        <f>D23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Paid Parents Retained from Prior Year</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="4">
+        <f>B22*(1-Assumptions!C10)</f>
+        <v/>
+      </c>
+      <c r="D25" s="4">
+        <f>C26*(1-Assumptions!C10)</f>
+        <v/>
+      </c>
+      <c r="E25" s="4">
+        <f>D24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Paid Coaches Retained from Prior Year</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="4">
+        <f>B23*(1-Assumptions!C10)</f>
+        <v/>
+      </c>
+      <c r="D26" s="4">
+        <f>C27*(1-Assumptions!C10)</f>
+        <v/>
+      </c>
+      <c r="E26" s="4">
+        <f>D25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Total Active Paid Parents</t>
+        </is>
+      </c>
+      <c r="B27" s="4">
+        <f>B22+B24</f>
+        <v/>
+      </c>
+      <c r="C27" s="4">
+        <f>C22+C24</f>
+        <v/>
+      </c>
+      <c r="D27" s="4">
+        <f>D22+D24</f>
+        <v/>
+      </c>
+      <c r="E27" s="4">
+        <f>D26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Total Active Paid Coaches</t>
+        </is>
+      </c>
+      <c r="B28" s="6">
+        <f>B23+B25</f>
+        <v/>
+      </c>
+      <c r="C28" s="6">
+        <f>C23+C25</f>
+        <v/>
+      </c>
+      <c r="D28" s="6">
+        <f>D23+D25</f>
+        <v/>
+      </c>
+      <c r="E28" s="6">
+        <f>D27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Parent App Revenue</t>
+        </is>
+      </c>
+      <c r="B29" s="6">
+        <f>B26*Assumptions!C11</f>
+        <v/>
+      </c>
+      <c r="C29" s="6">
+        <f>C26*Assumptions!C11</f>
+        <v/>
+      </c>
+      <c r="D29" s="6">
+        <f>D26*Assumptions!C11</f>
+        <v/>
+      </c>
+      <c r="E29" s="6">
+        <f>D28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Coach App Revenue</t>
+        </is>
+      </c>
+      <c r="B30" s="6">
+        <f>B27*Assumptions!C11</f>
+        <v/>
+      </c>
+      <c r="C30" s="6">
+        <f>C27*Assumptions!C11</f>
+        <v/>
+      </c>
+      <c r="D30" s="6">
+        <f>D27*Assumptions!C11</f>
+        <v/>
+      </c>
+      <c r="E30" s="6">
+        <f>D29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Total ARR</t>
+        </is>
+      </c>
+      <c r="B31" s="6">
+        <f>B28+B29</f>
+        <v/>
+      </c>
+      <c r="C31" s="6">
+        <f>C28+C29</f>
+        <v/>
+      </c>
+      <c r="D31" s="6">
+        <f>D28+D29</f>
+        <v/>
+      </c>
+      <c r="E31" s="6">
+        <f>D30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>Total MRR (Avg Year 3)</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr"/>
-      <c r="C22" s="6" t="inlineStr"/>
-      <c r="D22" s="6">
-        <f>D21/12</f>
-        <v/>
-      </c>
-      <c r="E22" s="6" t="inlineStr"/>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32">
+        <f>D30/12</f>
+        <v/>
+      </c>
+      <c r="E32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3225,7 +3405,7 @@
         <v/>
       </c>
       <c r="E3" s="6">
-        <f>County_League_Model!D21 / (County_League_Model!D13 + County_League_Model!D14 + County_League_Model!D15)</f>
+        <f>Funnel_Model!D30 / (Funnel_Model!D26 + Funnel_Model!D27)</f>
         <v/>
       </c>
     </row>
@@ -3599,7 +3779,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="6">
-        <f>IF(A4&lt;=12, (County_League_Model!B21/12)*(A4/12), IF(A4&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A4&lt;=12, (Funnel_Model!B30/12)*(A4/12), IF(A4&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E4" s="6">
@@ -3664,7 +3844,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="6">
-        <f>IF(A5&lt;=12, (County_League_Model!B21/12)*(A5/12), IF(A5&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A5&lt;=12, (Funnel_Model!B30/12)*(A5/12), IF(A5&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E5" s="6">
@@ -3729,7 +3909,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="6">
-        <f>IF(A6&lt;=12, (County_League_Model!B21/12)*(A6/12), IF(A6&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A6&lt;=12, (Funnel_Model!B30/12)*(A6/12), IF(A6&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E6" s="6">
@@ -3785,7 +3965,7 @@
         <v>0</v>
       </c>
       <c r="D7" s="6">
-        <f>IF(A7&lt;=12, (County_League_Model!B21/12)*(A7/12), IF(A7&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A7&lt;=12, (Funnel_Model!B30/12)*(A7/12), IF(A7&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E7" s="6">
@@ -3850,7 +4030,7 @@
         <v>0</v>
       </c>
       <c r="D8" s="6">
-        <f>IF(A8&lt;=12, (County_League_Model!B21/12)*(A8/12), IF(A8&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A8&lt;=12, (Funnel_Model!B30/12)*(A8/12), IF(A8&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E8" s="6">
@@ -3915,7 +4095,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="6">
-        <f>IF(A9&lt;=12, (County_League_Model!B21/12)*(A9/12), IF(A9&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A9&lt;=12, (Funnel_Model!B30/12)*(A9/12), IF(A9&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E9" s="6">
@@ -3971,7 +4151,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="6">
-        <f>IF(A10&lt;=12, (County_League_Model!B21/12)*(A10/12), IF(A10&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A10&lt;=12, (Funnel_Model!B30/12)*(A10/12), IF(A10&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E10" s="6">
@@ -4027,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="6">
-        <f>IF(A11&lt;=12, (County_League_Model!B21/12)*(A11/12), IF(A11&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A11&lt;=12, (Funnel_Model!B30/12)*(A11/12), IF(A11&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E11" s="6">
@@ -4084,7 +4264,7 @@
         <v/>
       </c>
       <c r="D12" s="6">
-        <f>IF(A12&lt;=12, (County_League_Model!B21/12)*(A12/12), IF(A12&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A12&lt;=12, (Funnel_Model!B30/12)*(A12/12), IF(A12&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E12" s="6">
@@ -4140,7 +4320,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="6">
-        <f>IF(A13&lt;=12, (County_League_Model!B21/12)*(A13/12), IF(A13&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A13&lt;=12, (Funnel_Model!B30/12)*(A13/12), IF(A13&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E13" s="6">
@@ -4196,7 +4376,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="6">
-        <f>IF(A14&lt;=12, (County_League_Model!B21/12)*(A14/12), IF(A14&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A14&lt;=12, (Funnel_Model!B30/12)*(A14/12), IF(A14&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E14" s="6">
@@ -4252,7 +4432,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="6">
-        <f>IF(A15&lt;=12, (County_League_Model!B21/12)*(A15/12), IF(A15&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A15&lt;=12, (Funnel_Model!B30/12)*(A15/12), IF(A15&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E15" s="6">
@@ -4308,7 +4488,7 @@
         <v>0</v>
       </c>
       <c r="D16" s="6">
-        <f>IF(A16&lt;=12, (County_League_Model!B21/12)*(A16/12), IF(A16&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A16&lt;=12, (Funnel_Model!B30/12)*(A16/12), IF(A16&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E16" s="6">
@@ -4364,7 +4544,7 @@
         <v>0</v>
       </c>
       <c r="D17" s="6">
-        <f>IF(A17&lt;=12, (County_League_Model!B21/12)*(A17/12), IF(A17&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A17&lt;=12, (Funnel_Model!B30/12)*(A17/12), IF(A17&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E17" s="6">
@@ -4420,7 +4600,7 @@
         <v>0</v>
       </c>
       <c r="D18" s="6">
-        <f>IF(A18&lt;=12, (County_League_Model!B21/12)*(A18/12), IF(A18&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A18&lt;=12, (Funnel_Model!B30/12)*(A18/12), IF(A18&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E18" s="6">
@@ -4476,7 +4656,7 @@
         <v>0</v>
       </c>
       <c r="D19" s="6">
-        <f>IF(A19&lt;=12, (County_League_Model!B21/12)*(A19/12), IF(A19&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A19&lt;=12, (Funnel_Model!B30/12)*(A19/12), IF(A19&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E19" s="6">
@@ -4532,7 +4712,7 @@
         <v>0</v>
       </c>
       <c r="D20" s="6">
-        <f>IF(A20&lt;=12, (County_League_Model!B21/12)*(A20/12), IF(A20&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A20&lt;=12, (Funnel_Model!B30/12)*(A20/12), IF(A20&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E20" s="6">
@@ -4588,7 +4768,7 @@
         <v>0</v>
       </c>
       <c r="D21" s="6">
-        <f>IF(A21&lt;=12, (County_League_Model!B21/12)*(A21/12), IF(A21&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A21&lt;=12, (Funnel_Model!B30/12)*(A21/12), IF(A21&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E21" s="6">
@@ -4644,7 +4824,7 @@
         <v>0</v>
       </c>
       <c r="D22" s="6">
-        <f>IF(A22&lt;=12, (County_League_Model!B21/12)*(A22/12), IF(A22&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A22&lt;=12, (Funnel_Model!B30/12)*(A22/12), IF(A22&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E22" s="6">
@@ -4700,7 +4880,7 @@
         <v>0</v>
       </c>
       <c r="D23" s="6">
-        <f>IF(A23&lt;=12, (County_League_Model!B21/12)*(A23/12), IF(A23&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A23&lt;=12, (Funnel_Model!B30/12)*(A23/12), IF(A23&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E23" s="6">
@@ -4757,7 +4937,7 @@
         <v/>
       </c>
       <c r="D24" s="6">
-        <f>IF(A24&lt;=12, (County_League_Model!B21/12)*(A24/12), IF(A24&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A24&lt;=12, (Funnel_Model!B30/12)*(A24/12), IF(A24&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E24" s="6">
@@ -4813,7 +4993,7 @@
         <v>0</v>
       </c>
       <c r="D25" s="6">
-        <f>IF(A25&lt;=12, (County_League_Model!B21/12)*(A25/12), IF(A25&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A25&lt;=12, (Funnel_Model!B30/12)*(A25/12), IF(A25&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E25" s="6">
@@ -4869,7 +5049,7 @@
         <v>0</v>
       </c>
       <c r="D26" s="6">
-        <f>IF(A26&lt;=12, (County_League_Model!B21/12)*(A26/12), IF(A26&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A26&lt;=12, (Funnel_Model!B30/12)*(A26/12), IF(A26&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E26" s="6">
@@ -4925,7 +5105,7 @@
         <v>0</v>
       </c>
       <c r="D27" s="6">
-        <f>IF(A27&lt;=12, (County_League_Model!B21/12)*(A27/12), IF(A27&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A27&lt;=12, (Funnel_Model!B30/12)*(A27/12), IF(A27&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E27" s="6">
@@ -4981,7 +5161,7 @@
         <v>0</v>
       </c>
       <c r="D28" s="6">
-        <f>IF(A28&lt;=12, (County_League_Model!B21/12)*(A28/12), IF(A28&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A28&lt;=12, (Funnel_Model!B30/12)*(A28/12), IF(A28&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E28" s="6">
@@ -5037,7 +5217,7 @@
         <v>0</v>
       </c>
       <c r="D29" s="6">
-        <f>IF(A29&lt;=12, (County_League_Model!B21/12)*(A29/12), IF(A29&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A29&lt;=12, (Funnel_Model!B30/12)*(A29/12), IF(A29&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E29" s="6">
@@ -5093,7 +5273,7 @@
         <v>0</v>
       </c>
       <c r="D30" s="6">
-        <f>IF(A30&lt;=12, (County_League_Model!B21/12)*(A30/12), IF(A30&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A30&lt;=12, (Funnel_Model!B30/12)*(A30/12), IF(A30&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E30" s="6">
@@ -5149,7 +5329,7 @@
         <v>0</v>
       </c>
       <c r="D31" s="6">
-        <f>IF(A31&lt;=12, (County_League_Model!B21/12)*(A31/12), IF(A31&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A31&lt;=12, (Funnel_Model!B30/12)*(A31/12), IF(A31&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E31" s="6">
@@ -5205,7 +5385,7 @@
         <v>0</v>
       </c>
       <c r="D32" s="6">
-        <f>IF(A32&lt;=12, (County_League_Model!B21/12)*(A32/12), IF(A32&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A32&lt;=12, (Funnel_Model!B30/12)*(A32/12), IF(A32&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E32" s="6">
@@ -5261,7 +5441,7 @@
         <v>0</v>
       </c>
       <c r="D33" s="6">
-        <f>IF(A33&lt;=12, (County_League_Model!B21/12)*(A33/12), IF(A33&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A33&lt;=12, (Funnel_Model!B30/12)*(A33/12), IF(A33&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E33" s="6">
@@ -5317,7 +5497,7 @@
         <v>0</v>
       </c>
       <c r="D34" s="6">
-        <f>IF(A34&lt;=12, (County_League_Model!B21/12)*(A34/12), IF(A34&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A34&lt;=12, (Funnel_Model!B30/12)*(A34/12), IF(A34&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E34" s="6">
@@ -5373,7 +5553,7 @@
         <v>0</v>
       </c>
       <c r="D35" s="6">
-        <f>IF(A35&lt;=12, (County_League_Model!B21/12)*(A35/12), IF(A35&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A35&lt;=12, (Funnel_Model!B30/12)*(A35/12), IF(A35&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E35" s="6">
@@ -5429,7 +5609,7 @@
         <v>0</v>
       </c>
       <c r="D36" s="6">
-        <f>IF(A36&lt;=12, (County_League_Model!B21/12)*(A36/12), IF(A36&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A36&lt;=12, (Funnel_Model!B30/12)*(A36/12), IF(A36&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E36" s="6">
@@ -5485,7 +5665,7 @@
         <v>0</v>
       </c>
       <c r="D37" s="6">
-        <f>IF(A37&lt;=12, (County_League_Model!B21/12)*(A37/12), IF(A37&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A37&lt;=12, (Funnel_Model!B30/12)*(A37/12), IF(A37&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E37" s="6">
@@ -5541,7 +5721,7 @@
         <v>0</v>
       </c>
       <c r="D38" s="6">
-        <f>IF(A38&lt;=12, (County_League_Model!B21/12)*(A38/12), IF(A38&lt;=24, (County_League_Model!C21/12), (County_League_Model!D21/12)))</f>
+        <f>IF(A38&lt;=12, (Funnel_Model!B30/12)*(A38/12), IF(A38&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
         <v/>
       </c>
       <c r="E38" s="6">
@@ -5722,7 +5902,7 @@
         </is>
       </c>
       <c r="B8" s="6">
-        <f>County_League_Model!D22</f>
+        <f>Funnel_Model!D31</f>
         <v/>
       </c>
       <c r="C8" s="6" t="n"/>
@@ -5885,9 +6065,8 @@
       <c r="D5" t="n">
         <v>5</v>
       </c>
-      <c r="E5">
-        <f>County_League_Model!B5</f>
-        <v/>
+      <c r="E5" t="n">
+        <v>0</v>
       </c>
       <c r="F5">
         <f>IF(E5&gt;=D5,"Met","Pending")</f>
@@ -5914,7 +6093,7 @@
         <v>4000</v>
       </c>
       <c r="E6">
-        <f>County_League_Model!D22</f>
+        <f>Funnel_Model!D31</f>
         <v/>
       </c>
       <c r="F6">
@@ -5970,7 +6149,7 @@
         <v>35000</v>
       </c>
       <c r="E8" s="5">
-        <f>County_League_Model!D22</f>
+        <f>Funnel_Model!D31</f>
         <v/>
       </c>
       <c r="F8">
@@ -6084,7 +6263,7 @@
         <v>100000</v>
       </c>
       <c r="E12">
-        <f>County_League_Model!D22</f>
+        <f>Funnel_Model!D31</f>
         <v/>
       </c>
       <c r="F12">
@@ -6111,9 +6290,8 @@
       <c r="D13" t="n">
         <v>10</v>
       </c>
-      <c r="E13">
-        <f>County_League_Model!D15</f>
-        <v/>
+      <c r="E13" t="n">
+        <v>0</v>
       </c>
       <c r="F13">
         <f>IF(E13&gt;=D13,"Met","Pending")</f>

</xml_diff>

<commit_message>
Add investor-ready improvements: Financial_Summary tab (capital-to-ARR), KPI_Summary tab (quarterly metrics), Funding_Overview tab (timeline), milestone dates in Milestones tab, and formatted Pay_Triggers as OpEx section
</commit_message>
<xml_diff>
--- a/use-of-funds/BLU Use-of-Funds Model.xlsx
+++ b/use-of-funds/BLU Use-of-Funds Model.xlsx
@@ -20,6 +20,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios_Output" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales_Comp" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infra_Estimates" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial_Summary" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI_Summary" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding_Overview" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,9 +31,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -95,7 +99,7 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -109,6 +113,8 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="3"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="4"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1216,6 +1222,691 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Financial Summary - Capital Efficiency</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Tranche</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Capital Invested</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Projected ARR</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Projected MRR</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Capital-to-ARR Ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tranche A</t>
+        </is>
+      </c>
+      <c r="B3" s="6">
+        <f>Assumptions!C30</f>
+        <v/>
+      </c>
+      <c r="C3" s="6">
+        <f>Funnel_Model!B30</f>
+        <v/>
+      </c>
+      <c r="D3" s="6">
+        <f>Funnel_Model!B30/12</f>
+        <v/>
+      </c>
+      <c r="E3" s="11">
+        <f>B3/C3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Tranche B</t>
+        </is>
+      </c>
+      <c r="B4" s="6">
+        <f>Assumptions!C30+Assumptions!C31</f>
+        <v/>
+      </c>
+      <c r="C4" s="6">
+        <f>Funnel_Model!C30</f>
+        <v/>
+      </c>
+      <c r="D4" s="6">
+        <f>Funnel_Model!C30/12</f>
+        <v/>
+      </c>
+      <c r="E4" s="11">
+        <f>B4/C4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Tranche C</t>
+        </is>
+      </c>
+      <c r="B5" s="6">
+        <f>Assumptions!C30+Assumptions!C31+Assumptions!C32</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>Funnel_Model!D30</f>
+        <v/>
+      </c>
+      <c r="D5" s="6">
+        <f>Funnel_Model!D30/12</f>
+        <v/>
+      </c>
+      <c r="E5" s="11">
+        <f>B5/C5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" s="6" t="inlineStr"/>
+      <c r="C6" s="6" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr"/>
+      <c r="E6" s="11" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B7" s="6">
+        <f>B5</f>
+        <v/>
+      </c>
+      <c r="C7" s="6">
+        <f>C5</f>
+        <v/>
+      </c>
+      <c r="D7" s="6">
+        <f>D5</f>
+        <v/>
+      </c>
+      <c r="E7" s="11">
+        <f>B7/C7</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KPI Summary - Quarterly Metrics</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Year 1 Avg</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Year 2 Avg</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Year 3 Avg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>U-CAC ($/umpire)</t>
+        </is>
+      </c>
+      <c r="B3" s="5">
+        <f>Assumptions!C17</f>
+        <v/>
+      </c>
+      <c r="C3" s="5">
+        <f>Assumptions!C17</f>
+        <v/>
+      </c>
+      <c r="D3" s="5">
+        <f>Assumptions!C17</f>
+        <v/>
+      </c>
+      <c r="E3" s="5">
+        <f>Assumptions!C17</f>
+        <v/>
+      </c>
+      <c r="F3" s="5">
+        <f>Assumptions!C17</f>
+        <v/>
+      </c>
+      <c r="G3" s="5">
+        <f>Assumptions!C17</f>
+        <v/>
+      </c>
+      <c r="H3" s="5">
+        <f>Assumptions!C17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Parent Conversion %</t>
+        </is>
+      </c>
+      <c r="B4" s="5">
+        <f>Assumptions!C8</f>
+        <v/>
+      </c>
+      <c r="C4" s="5">
+        <f>Assumptions!C8</f>
+        <v/>
+      </c>
+      <c r="D4" s="5">
+        <f>Assumptions!C8</f>
+        <v/>
+      </c>
+      <c r="E4" s="5">
+        <f>Assumptions!C8</f>
+        <v/>
+      </c>
+      <c r="F4" s="5">
+        <f>Assumptions!C8</f>
+        <v/>
+      </c>
+      <c r="G4" s="5">
+        <f>Assumptions!C8</f>
+        <v/>
+      </c>
+      <c r="H4" s="5">
+        <f>Assumptions!C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Coach Conversion %</t>
+        </is>
+      </c>
+      <c r="B5" s="6">
+        <f>Assumptions!C9</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>Assumptions!C9</f>
+        <v/>
+      </c>
+      <c r="D5" s="6">
+        <f>Assumptions!C9</f>
+        <v/>
+      </c>
+      <c r="E5" s="6">
+        <f>Assumptions!C9</f>
+        <v/>
+      </c>
+      <c r="F5" s="6">
+        <f>Assumptions!C9</f>
+        <v/>
+      </c>
+      <c r="G5" s="6">
+        <f>Assumptions!C9</f>
+        <v/>
+      </c>
+      <c r="H5" s="6">
+        <f>Assumptions!C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ARPU (Annual)</t>
+        </is>
+      </c>
+      <c r="B6" s="6">
+        <f>Assumptions!C11</f>
+        <v/>
+      </c>
+      <c r="C6" s="6">
+        <f>Assumptions!C11</f>
+        <v/>
+      </c>
+      <c r="D6" s="6">
+        <f>Assumptions!C11</f>
+        <v/>
+      </c>
+      <c r="E6" s="6">
+        <f>Assumptions!C11</f>
+        <v/>
+      </c>
+      <c r="F6" s="6">
+        <f>Assumptions!C11</f>
+        <v/>
+      </c>
+      <c r="G6" s="6">
+        <f>Assumptions!C11</f>
+        <v/>
+      </c>
+      <c r="H6" s="6">
+        <f>Unit_Economics!E3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LTV</t>
+        </is>
+      </c>
+      <c r="B7" s="11">
+        <f>Unit_Economics!B7</f>
+        <v/>
+      </c>
+      <c r="C7" s="11">
+        <f>Unit_Economics!B7</f>
+        <v/>
+      </c>
+      <c r="D7" s="11">
+        <f>Unit_Economics!B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="11">
+        <f>Unit_Economics!B7</f>
+        <v/>
+      </c>
+      <c r="F7" s="11">
+        <f>Unit_Economics!B7</f>
+        <v/>
+      </c>
+      <c r="G7" s="11">
+        <f>Unit_Economics!B7</f>
+        <v/>
+      </c>
+      <c r="H7" s="11">
+        <f>Unit_Economics!E7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LTV/CAC Ratio</t>
+        </is>
+      </c>
+      <c r="B8" s="12">
+        <f>Unit_Economics!B10</f>
+        <v/>
+      </c>
+      <c r="C8" s="12">
+        <f>Unit_Economics!B10</f>
+        <v/>
+      </c>
+      <c r="D8" s="12">
+        <f>Unit_Economics!B10</f>
+        <v/>
+      </c>
+      <c r="E8" s="12">
+        <f>Unit_Economics!B10</f>
+        <v/>
+      </c>
+      <c r="F8" s="12">
+        <f>Unit_Economics!B10</f>
+        <v/>
+      </c>
+      <c r="G8" s="12">
+        <f>Unit_Economics!B10</f>
+        <v/>
+      </c>
+      <c r="H8" s="12">
+        <f>Unit_Economics!E10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Payback Period (Months)</t>
+        </is>
+      </c>
+      <c r="B9" s="5">
+        <f>Unit_Economics!B11</f>
+        <v/>
+      </c>
+      <c r="C9" s="5">
+        <f>Unit_Economics!B11</f>
+        <v/>
+      </c>
+      <c r="D9" s="5">
+        <f>Unit_Economics!B11</f>
+        <v/>
+      </c>
+      <c r="E9" s="5">
+        <f>Unit_Economics!B11</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>Unit_Economics!B11</f>
+        <v/>
+      </c>
+      <c r="G9" s="5">
+        <f>Unit_Economics!B11</f>
+        <v/>
+      </c>
+      <c r="H9" s="5">
+        <f>Unit_Economics!E11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Gross Margin</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>Assumptions!C15</f>
+        <v/>
+      </c>
+      <c r="C10">
+        <f>Assumptions!C15</f>
+        <v/>
+      </c>
+      <c r="D10">
+        <f>Assumptions!C15</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>Assumptions!C15</f>
+        <v/>
+      </c>
+      <c r="F10">
+        <f>Assumptions!C15</f>
+        <v/>
+      </c>
+      <c r="G10">
+        <f>Assumptions!C15</f>
+        <v/>
+      </c>
+      <c r="H10">
+        <f>Assumptions!C15</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Funding Overview - Timeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Tranche</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>End Date</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Major Deliverable</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tranche A → MVP</t>
+        </is>
+      </c>
+      <c r="B3" s="6">
+        <f>Assumptions!C30</f>
+        <v/>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Jan 2025</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sep 2025</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>9 months</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Umpire MVP, 100+ umpires, $3-5k MRR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Tranche B → Pilot Scale</t>
+        </is>
+      </c>
+      <c r="B4" s="6">
+        <f>Assumptions!C31</f>
+        <v/>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Jan 2026</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>12 months</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>$35k MRR, 2% parent / 3% coach conversion</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Tranche C → Growth</t>
+        </is>
+      </c>
+      <c r="B5" s="6">
+        <f>Assumptions!C32</f>
+        <v/>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Jan 2027</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Dec 2027</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>12 months</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>$100k MRR, scalable B2C engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B7" s="6">
+        <f>Assumptions!C30+Assumptions!C31+Assumptions!C32</f>
+        <v/>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>33 months</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -5789,7 +6480,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Founder Pay Triggers</t>
+          <t>Founder Compensation (OpEx)</t>
         </is>
       </c>
     </row>
@@ -5801,22 +6492,22 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Annual Salary (per Founder)</t>
+          <t>MRR Trigger</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>MRR Trigger</t>
+          <t>Per-Founder Annual</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Tranche Trigger</t>
+          <t>Combined Annual Cost</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Monthly Impact</t>
         </is>
       </c>
     </row>
@@ -5824,22 +6515,20 @@
       <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="6">
         <f>Assumptions!C22</f>
         <v/>
       </c>
-      <c r="C3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Tranche A</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>MVP &amp; Pilot Phase</t>
-        </is>
+      <c r="D3" s="6">
+        <f>Assumptions!C22*2</f>
+        <v/>
+      </c>
+      <c r="E3" s="6">
+        <f>Assumptions!C22*2/12</f>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -5847,22 +6536,20 @@
         <v>2</v>
       </c>
       <c r="B4" s="6">
+        <f>Assumptions!C25</f>
+        <v/>
+      </c>
+      <c r="C4" s="6">
         <f>Assumptions!C23</f>
         <v/>
       </c>
-      <c r="C4" s="6">
-        <f>Assumptions!C25</f>
-        <v/>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Tranche B</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>PMF Phase</t>
-        </is>
+      <c r="D4" s="6">
+        <f>Assumptions!C23*2</f>
+        <v/>
+      </c>
+      <c r="E4" s="6">
+        <f>Assumptions!C23*2/12</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -5870,65 +6557,32 @@
         <v>3</v>
       </c>
       <c r="B5" s="6">
+        <f>Assumptions!C26</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
         <f>Assumptions!C24</f>
         <v/>
       </c>
-      <c r="C5" s="6">
-        <f>Assumptions!C26</f>
-        <v/>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Tranche C</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Scale Phase</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Current Status</t>
-        </is>
+      <c r="D5" s="6">
+        <f>Assumptions!C24*2</f>
+        <v/>
+      </c>
+      <c r="E5" s="6">
+        <f>Assumptions!C24*2/12</f>
+        <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Current MRR</t>
-        </is>
-      </c>
-      <c r="B8" s="6">
-        <f>Funnel_Model!D31</f>
-        <v/>
-      </c>
+      <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Current Annual Pay (per)</t>
-        </is>
-      </c>
-      <c r="B9" s="6">
-        <f>IF(B8&gt;=C4, B4, IF(B8&gt;=C3, B3, B2))</f>
-        <v/>
-      </c>
+      <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Total Founder Payroll (Annual)</t>
-        </is>
-      </c>
-      <c r="B10" s="6">
-        <f>B9*2</f>
-        <v/>
-      </c>
+      <c r="B10" s="6" t="n"/>
       <c r="C10" s="6" t="n"/>
     </row>
   </sheetData>
@@ -5942,7 +6596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5991,6 +6645,11 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Completion Date</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6018,6 +6677,11 @@
         <f>IF(E3&gt;=D3,"Met","Pending")</f>
         <v/>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Apr 2025</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6045,6 +6709,11 @@
         <f>IF(E4&gt;=D4,"Met","Pending")</f>
         <v/>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Jun 2025</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6072,6 +6741,11 @@
         <f>IF(E5&gt;=D5,"Met","Pending")</f>
         <v/>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Jul 2025</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6100,6 +6774,11 @@
         <f>IF(E6&gt;=D6,"Met","Pending")</f>
         <v/>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Jan 2026</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6128,6 +6807,11 @@
         <f>IF(E7&gt;=D7,"Met","Pending")</f>
         <v/>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Jan 2026</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6156,6 +6840,11 @@
         <f>IF(E8&gt;=D8,"Met","Pending")</f>
         <v/>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6185,6 +6874,11 @@
         <f>IF(E9&gt;=D9,"Met","Pending")</f>
         <v/>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6214,6 +6908,11 @@
         <f>IF(E10&gt;=D10,"Met","Pending")</f>
         <v/>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6242,6 +6941,11 @@
         <f>IF(E11&gt;=D11,"Met","Pending")</f>
         <v/>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6270,6 +6974,11 @@
         <f>IF(E12&gt;=D12,"Met","Pending")</f>
         <v/>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Dec 2027</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6296,6 +7005,11 @@
       <c r="F13">
         <f>IF(E13&gt;=D13,"Met","Pending")</f>
         <v/>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Dec 2027</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix #VALUE! errors in Funnel_Model and Cash_Runway tabs: correct row references for inputs (rows 6-10), Total ARR (row 31), Total Active Paid Users (rows 27-28), MRR (row 32), and revenue formulas
</commit_message>
<xml_diff>
--- a/use-of-funds/BLU Use-of-Funds Model.xlsx
+++ b/use-of-funds/BLU Use-of-Funds Model.xlsx
@@ -831,15 +831,15 @@
         </is>
       </c>
       <c r="B3" s="6">
-        <f>(Funnel_Model!D26*Scenarios!B3*Assumptions!D11) + (Funnel_Model!D27*Scenarios!B4*Assumptions!D11)</f>
+        <f>(Funnel_Model!D27*Scenarios!B3*Assumptions!D11) + (Funnel_Model!D28*Scenarios!B4*Assumptions!D11)</f>
         <v/>
       </c>
       <c r="C3" s="6">
-        <f>Funnel_Model!D30</f>
+        <f>Funnel_Model!D31</f>
         <v/>
       </c>
       <c r="D3" s="6">
-        <f>(Funnel_Model!D26*Scenarios!D3*Assumptions!E11) + (Funnel_Model!D27*Scenarios!D4*Assumptions!E11)</f>
+        <f>(Funnel_Model!D27*Scenarios!D3*Assumptions!E11) + (Funnel_Model!D28*Scenarios!D4*Assumptions!E11)</f>
         <v/>
       </c>
     </row>
@@ -850,15 +850,15 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>(Funnel_Model!D26*Scenarios!B3) + (Funnel_Model!D27*Scenarios!B4)</f>
+        <f>(Funnel_Model!D27*Scenarios!B3) + (Funnel_Model!D28*Scenarios!B4)</f>
         <v/>
       </c>
       <c r="C4" s="4">
-        <f>Funnel_Model!D26 + Funnel_Model!D27</f>
+        <f>Funnel_Model!D27 + Funnel_Model!D28</f>
         <v/>
       </c>
       <c r="D4" s="4">
-        <f>(Funnel_Model!D26*Scenarios!D3) + (Funnel_Model!D27*Scenarios!D4)</f>
+        <f>(Funnel_Model!D27*Scenarios!D3) + (Funnel_Model!D28*Scenarios!D4)</f>
         <v/>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>E6/Funnel_Model!C30</f>
+        <f>E6/Funnel_Model!C31</f>
         <v/>
       </c>
     </row>
@@ -1283,11 +1283,11 @@
         <v/>
       </c>
       <c r="C3" s="6">
-        <f>Funnel_Model!B30</f>
+        <f>Funnel_Model!B31</f>
         <v/>
       </c>
       <c r="D3" s="6">
-        <f>Funnel_Model!B30/12</f>
+        <f>Funnel_Model!B31/12</f>
         <v/>
       </c>
       <c r="E3" s="11">
@@ -1306,11 +1306,11 @@
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>Funnel_Model!C30</f>
+        <f>Funnel_Model!C31</f>
         <v/>
       </c>
       <c r="D4" s="6">
-        <f>Funnel_Model!C30/12</f>
+        <f>Funnel_Model!C31/12</f>
         <v/>
       </c>
       <c r="E4" s="11">
@@ -1329,11 +1329,11 @@
         <v/>
       </c>
       <c r="C5" s="6">
-        <f>Funnel_Model!D30</f>
+        <f>Funnel_Model!D31</f>
         <v/>
       </c>
       <c r="D5" s="6">
-        <f>Funnel_Model!D30/12</f>
+        <f>Funnel_Model!D31/12</f>
         <v/>
       </c>
       <c r="E5" s="11">
@@ -3639,15 +3639,15 @@
         </is>
       </c>
       <c r="B15" s="4">
-        <f>B8</f>
+        <f>B6</f>
         <v/>
       </c>
       <c r="C15" s="4">
-        <f>C8</f>
+        <f>C6</f>
         <v/>
       </c>
       <c r="D15" s="4">
-        <f>D8</f>
+        <f>D6</f>
         <v/>
       </c>
       <c r="E15" s="4">
@@ -3665,11 +3665,11 @@
         <v>0</v>
       </c>
       <c r="C16" s="4">
-        <f>B14*(1-B9)</f>
+        <f>B14*(1-B7)</f>
         <v/>
       </c>
       <c r="D16" s="4">
-        <f>C16*(1-C9)</f>
+        <f>C16*(1-C7)</f>
         <v/>
       </c>
       <c r="E16" s="4">
@@ -3707,15 +3707,15 @@
         </is>
       </c>
       <c r="B18" s="4">
-        <f>B16*B10</f>
+        <f>B16*B8</f>
         <v/>
       </c>
       <c r="C18" s="4">
-        <f>C16*C10</f>
+        <f>C16*C8</f>
         <v/>
       </c>
       <c r="D18" s="4">
-        <f>D16*D10</f>
+        <f>D16*D8</f>
         <v/>
       </c>
       <c r="E18" s="4">
@@ -3730,15 +3730,15 @@
         </is>
       </c>
       <c r="B19" s="4">
-        <f>B17*B11</f>
+        <f>B17*B9</f>
         <v/>
       </c>
       <c r="C19" s="4">
-        <f>C17*C11</f>
+        <f>C17*C9</f>
         <v/>
       </c>
       <c r="D19" s="4">
-        <f>D17*D11</f>
+        <f>D17*D9</f>
         <v/>
       </c>
       <c r="E19" s="4">
@@ -3753,15 +3753,15 @@
         </is>
       </c>
       <c r="B20">
-        <f>B18*B12</f>
+        <f>B18*B10</f>
         <v/>
       </c>
       <c r="C20">
-        <f>C18*C12</f>
+        <f>C18*C10</f>
         <v/>
       </c>
       <c r="D20">
-        <f>D18*D12</f>
+        <f>D18*D10</f>
         <v/>
       </c>
       <c r="E20">
@@ -3992,19 +3992,19 @@
         </is>
       </c>
       <c r="B31" s="6">
-        <f>B28+B29</f>
+        <f>B29+B30</f>
         <v/>
       </c>
       <c r="C31" s="6">
-        <f>C28+C29</f>
+        <f>C29+C30</f>
         <v/>
       </c>
       <c r="D31" s="6">
-        <f>D28+D29</f>
+        <f>D29+D30</f>
         <v/>
       </c>
       <c r="E31" s="6">
-        <f>D30</f>
+        <f>D31</f>
         <v/>
       </c>
     </row>
@@ -4017,7 +4017,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32">
-        <f>D30/12</f>
+        <f>D31/12</f>
         <v/>
       </c>
       <c r="E32" t="inlineStr"/>
@@ -4096,7 +4096,7 @@
         <v/>
       </c>
       <c r="E3" s="6">
-        <f>Funnel_Model!D30 / (Funnel_Model!D26 + Funnel_Model!D27)</f>
+        <f>Funnel_Model!D31 / (Funnel_Model!D27 + Funnel_Model!D28)</f>
         <v/>
       </c>
     </row>
@@ -4470,7 +4470,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="6">
-        <f>IF(A4&lt;=12, (Funnel_Model!B30/12)*(A4/12), IF(A4&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A4&lt;=12, (Funnel_Model!B31/12)*(A4/12), IF(A4&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E4" s="6">
@@ -4535,7 +4535,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="6">
-        <f>IF(A5&lt;=12, (Funnel_Model!B30/12)*(A5/12), IF(A5&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A5&lt;=12, (Funnel_Model!B31/12)*(A5/12), IF(A5&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E5" s="6">
@@ -4600,7 +4600,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="6">
-        <f>IF(A6&lt;=12, (Funnel_Model!B30/12)*(A6/12), IF(A6&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A6&lt;=12, (Funnel_Model!B31/12)*(A6/12), IF(A6&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E6" s="6">
@@ -4656,7 +4656,7 @@
         <v>0</v>
       </c>
       <c r="D7" s="6">
-        <f>IF(A7&lt;=12, (Funnel_Model!B30/12)*(A7/12), IF(A7&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A7&lt;=12, (Funnel_Model!B31/12)*(A7/12), IF(A7&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E7" s="6">
@@ -4721,7 +4721,7 @@
         <v>0</v>
       </c>
       <c r="D8" s="6">
-        <f>IF(A8&lt;=12, (Funnel_Model!B30/12)*(A8/12), IF(A8&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A8&lt;=12, (Funnel_Model!B31/12)*(A8/12), IF(A8&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E8" s="6">
@@ -4786,7 +4786,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="6">
-        <f>IF(A9&lt;=12, (Funnel_Model!B30/12)*(A9/12), IF(A9&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A9&lt;=12, (Funnel_Model!B31/12)*(A9/12), IF(A9&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E9" s="6">
@@ -4842,7 +4842,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="6">
-        <f>IF(A10&lt;=12, (Funnel_Model!B30/12)*(A10/12), IF(A10&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A10&lt;=12, (Funnel_Model!B31/12)*(A10/12), IF(A10&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E10" s="6">
@@ -4898,7 +4898,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="6">
-        <f>IF(A11&lt;=12, (Funnel_Model!B30/12)*(A11/12), IF(A11&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A11&lt;=12, (Funnel_Model!B31/12)*(A11/12), IF(A11&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E11" s="6">
@@ -4955,7 +4955,7 @@
         <v/>
       </c>
       <c r="D12" s="6">
-        <f>IF(A12&lt;=12, (Funnel_Model!B30/12)*(A12/12), IF(A12&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A12&lt;=12, (Funnel_Model!B31/12)*(A12/12), IF(A12&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E12" s="6">
@@ -5011,7 +5011,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="6">
-        <f>IF(A13&lt;=12, (Funnel_Model!B30/12)*(A13/12), IF(A13&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A13&lt;=12, (Funnel_Model!B31/12)*(A13/12), IF(A13&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E13" s="6">
@@ -5067,7 +5067,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="6">
-        <f>IF(A14&lt;=12, (Funnel_Model!B30/12)*(A14/12), IF(A14&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A14&lt;=12, (Funnel_Model!B31/12)*(A14/12), IF(A14&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E14" s="6">
@@ -5123,7 +5123,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="6">
-        <f>IF(A15&lt;=12, (Funnel_Model!B30/12)*(A15/12), IF(A15&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A15&lt;=12, (Funnel_Model!B31/12)*(A15/12), IF(A15&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E15" s="6">
@@ -5179,7 +5179,7 @@
         <v>0</v>
       </c>
       <c r="D16" s="6">
-        <f>IF(A16&lt;=12, (Funnel_Model!B30/12)*(A16/12), IF(A16&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A16&lt;=12, (Funnel_Model!B31/12)*(A16/12), IF(A16&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E16" s="6">
@@ -5235,7 +5235,7 @@
         <v>0</v>
       </c>
       <c r="D17" s="6">
-        <f>IF(A17&lt;=12, (Funnel_Model!B30/12)*(A17/12), IF(A17&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A17&lt;=12, (Funnel_Model!B31/12)*(A17/12), IF(A17&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E17" s="6">
@@ -5291,7 +5291,7 @@
         <v>0</v>
       </c>
       <c r="D18" s="6">
-        <f>IF(A18&lt;=12, (Funnel_Model!B30/12)*(A18/12), IF(A18&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A18&lt;=12, (Funnel_Model!B31/12)*(A18/12), IF(A18&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E18" s="6">
@@ -5347,7 +5347,7 @@
         <v>0</v>
       </c>
       <c r="D19" s="6">
-        <f>IF(A19&lt;=12, (Funnel_Model!B30/12)*(A19/12), IF(A19&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A19&lt;=12, (Funnel_Model!B31/12)*(A19/12), IF(A19&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E19" s="6">
@@ -5403,7 +5403,7 @@
         <v>0</v>
       </c>
       <c r="D20" s="6">
-        <f>IF(A20&lt;=12, (Funnel_Model!B30/12)*(A20/12), IF(A20&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A20&lt;=12, (Funnel_Model!B31/12)*(A20/12), IF(A20&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E20" s="6">
@@ -5459,7 +5459,7 @@
         <v>0</v>
       </c>
       <c r="D21" s="6">
-        <f>IF(A21&lt;=12, (Funnel_Model!B30/12)*(A21/12), IF(A21&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A21&lt;=12, (Funnel_Model!B31/12)*(A21/12), IF(A21&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E21" s="6">
@@ -5515,7 +5515,7 @@
         <v>0</v>
       </c>
       <c r="D22" s="6">
-        <f>IF(A22&lt;=12, (Funnel_Model!B30/12)*(A22/12), IF(A22&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A22&lt;=12, (Funnel_Model!B31/12)*(A22/12), IF(A22&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E22" s="6">
@@ -5571,7 +5571,7 @@
         <v>0</v>
       </c>
       <c r="D23" s="6">
-        <f>IF(A23&lt;=12, (Funnel_Model!B30/12)*(A23/12), IF(A23&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A23&lt;=12, (Funnel_Model!B31/12)*(A23/12), IF(A23&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E23" s="6">
@@ -5628,7 +5628,7 @@
         <v/>
       </c>
       <c r="D24" s="6">
-        <f>IF(A24&lt;=12, (Funnel_Model!B30/12)*(A24/12), IF(A24&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A24&lt;=12, (Funnel_Model!B31/12)*(A24/12), IF(A24&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E24" s="6">
@@ -5684,7 +5684,7 @@
         <v>0</v>
       </c>
       <c r="D25" s="6">
-        <f>IF(A25&lt;=12, (Funnel_Model!B30/12)*(A25/12), IF(A25&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A25&lt;=12, (Funnel_Model!B31/12)*(A25/12), IF(A25&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E25" s="6">
@@ -5740,7 +5740,7 @@
         <v>0</v>
       </c>
       <c r="D26" s="6">
-        <f>IF(A26&lt;=12, (Funnel_Model!B30/12)*(A26/12), IF(A26&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A26&lt;=12, (Funnel_Model!B31/12)*(A26/12), IF(A26&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E26" s="6">
@@ -5796,7 +5796,7 @@
         <v>0</v>
       </c>
       <c r="D27" s="6">
-        <f>IF(A27&lt;=12, (Funnel_Model!B30/12)*(A27/12), IF(A27&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A27&lt;=12, (Funnel_Model!B31/12)*(A27/12), IF(A27&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E27" s="6">
@@ -5852,7 +5852,7 @@
         <v>0</v>
       </c>
       <c r="D28" s="6">
-        <f>IF(A28&lt;=12, (Funnel_Model!B30/12)*(A28/12), IF(A28&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A28&lt;=12, (Funnel_Model!B31/12)*(A28/12), IF(A28&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E28" s="6">
@@ -5908,7 +5908,7 @@
         <v>0</v>
       </c>
       <c r="D29" s="6">
-        <f>IF(A29&lt;=12, (Funnel_Model!B30/12)*(A29/12), IF(A29&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A29&lt;=12, (Funnel_Model!B31/12)*(A29/12), IF(A29&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E29" s="6">
@@ -5964,7 +5964,7 @@
         <v>0</v>
       </c>
       <c r="D30" s="6">
-        <f>IF(A30&lt;=12, (Funnel_Model!B30/12)*(A30/12), IF(A30&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A30&lt;=12, (Funnel_Model!B31/12)*(A30/12), IF(A30&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E30" s="6">
@@ -6020,7 +6020,7 @@
         <v>0</v>
       </c>
       <c r="D31" s="6">
-        <f>IF(A31&lt;=12, (Funnel_Model!B30/12)*(A31/12), IF(A31&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A31&lt;=12, (Funnel_Model!B31/12)*(A31/12), IF(A31&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E31" s="6">
@@ -6076,7 +6076,7 @@
         <v>0</v>
       </c>
       <c r="D32" s="6">
-        <f>IF(A32&lt;=12, (Funnel_Model!B30/12)*(A32/12), IF(A32&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A32&lt;=12, (Funnel_Model!B31/12)*(A32/12), IF(A32&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E32" s="6">
@@ -6132,7 +6132,7 @@
         <v>0</v>
       </c>
       <c r="D33" s="6">
-        <f>IF(A33&lt;=12, (Funnel_Model!B30/12)*(A33/12), IF(A33&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A33&lt;=12, (Funnel_Model!B31/12)*(A33/12), IF(A33&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E33" s="6">
@@ -6188,7 +6188,7 @@
         <v>0</v>
       </c>
       <c r="D34" s="6">
-        <f>IF(A34&lt;=12, (Funnel_Model!B30/12)*(A34/12), IF(A34&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A34&lt;=12, (Funnel_Model!B31/12)*(A34/12), IF(A34&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E34" s="6">
@@ -6244,7 +6244,7 @@
         <v>0</v>
       </c>
       <c r="D35" s="6">
-        <f>IF(A35&lt;=12, (Funnel_Model!B30/12)*(A35/12), IF(A35&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A35&lt;=12, (Funnel_Model!B31/12)*(A35/12), IF(A35&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E35" s="6">
@@ -6300,7 +6300,7 @@
         <v>0</v>
       </c>
       <c r="D36" s="6">
-        <f>IF(A36&lt;=12, (Funnel_Model!B30/12)*(A36/12), IF(A36&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A36&lt;=12, (Funnel_Model!B31/12)*(A36/12), IF(A36&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E36" s="6">
@@ -6356,7 +6356,7 @@
         <v>0</v>
       </c>
       <c r="D37" s="6">
-        <f>IF(A37&lt;=12, (Funnel_Model!B30/12)*(A37/12), IF(A37&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A37&lt;=12, (Funnel_Model!B31/12)*(A37/12), IF(A37&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E37" s="6">
@@ -6412,7 +6412,7 @@
         <v>0</v>
       </c>
       <c r="D38" s="6">
-        <f>IF(A38&lt;=12, (Funnel_Model!B30/12)*(A38/12), IF(A38&lt;=24, (Funnel_Model!C30/12), (Funnel_Model!D30/12)))</f>
+        <f>IF(A38&lt;=12, (Funnel_Model!B31/12)*(A38/12), IF(A38&lt;=24, (Funnel_Model!C31/12), (Funnel_Model!D31/12)))</f>
         <v/>
       </c>
       <c r="E38" s="6">
@@ -6767,7 +6767,7 @@
         <v>4000</v>
       </c>
       <c r="E6">
-        <f>Funnel_Model!D31</f>
+        <f>Funnel_Model!D32</f>
         <v/>
       </c>
       <c r="F6">
@@ -6833,7 +6833,7 @@
         <v>35000</v>
       </c>
       <c r="E8" s="5">
-        <f>Funnel_Model!D31</f>
+        <f>Funnel_Model!D32</f>
         <v/>
       </c>
       <c r="F8">
@@ -6967,7 +6967,7 @@
         <v>100000</v>
       </c>
       <c r="E12">
-        <f>Funnel_Model!D31</f>
+        <f>Funnel_Model!D32</f>
         <v/>
       </c>
       <c r="F12">

</xml_diff>

<commit_message>
Fix #VALUE! errors: Remove header text from data columns in Funnel_Model (INPUTS, CALCULATIONS, Revenue sections). Headers now only in column A, preventing text from interfering with formulas.
</commit_message>
<xml_diff>
--- a/use-of-funds/BLU Use-of-Funds Model.xlsx
+++ b/use-of-funds/BLU Use-of-Funds Model.xlsx
@@ -3412,7 +3412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -3464,313 +3464,297 @@
       <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>INPUTS</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Year 1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Year 2</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Year 3</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>New Umpires Acquired</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C5" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D5" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Target from Umpire_Funnel tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Umpire Churn Rate</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Annual churn rate</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Avg. Games per Umpire per Year</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C7" t="n">
+        <v>20</v>
+      </c>
+      <c r="D7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Games captured annually</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>New Umpires Acquired</t>
+          <t>Avg. Unique Players per Game</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>1000</v>
+        <v>25</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>5000</v>
+        <v>25</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>15000</v>
+        <v>25</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Target from Umpire_Funnel tab</t>
+          <t>Players reached per game</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Umpire Churn Rate</t>
+          <t>Avg. Parents/Coaches per Player</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>0.2</v>
+        <v>1.5</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>0.2</v>
+        <v>1.5</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>0.2</v>
+        <v>1.5</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Annual churn rate</t>
+          <t>Parents &amp; coaches per player</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Avg. Games per Umpire per Year</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Games captured annually</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Avg. Unique Players per Game</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Players reached per game</t>
-        </is>
-      </c>
+          <t>CALCULATIONS</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr"/>
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Avg. Parents/Coaches per Player</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C12" s="9" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D12" s="9" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Parents &amp; coaches per player</t>
-        </is>
-      </c>
+      <c r="B12" s="9" t="n"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+      <c r="A13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CALCULATIONS</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Year 1</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Year 2</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Year 3</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
+          <t>New Umpires Acquired</t>
+        </is>
+      </c>
+      <c r="B14" s="4">
+        <f>B8</f>
+        <v/>
+      </c>
+      <c r="C14" s="4">
+        <f>C8</f>
+        <v/>
+      </c>
+      <c r="D14" s="4">
+        <f>D8</f>
+        <v/>
+      </c>
+      <c r="E14" s="4">
+        <f>D14</f>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>New Umpires Acquired</t>
-        </is>
-      </c>
-      <c r="B15" s="4">
-        <f>B6</f>
-        <v/>
+          <t>Umpires Retained from Prior Year</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="C15" s="4">
-        <f>C6</f>
+        <f>B14*(1-B9)</f>
         <v/>
       </c>
       <c r="D15" s="4">
-        <f>D6</f>
+        <f>C16*(1-C9)</f>
         <v/>
       </c>
       <c r="E15" s="4">
-        <f>D14</f>
+        <f>D15</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Umpires Retained from Prior Year</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>0</v>
+          <t>Total Active Umpires</t>
+        </is>
+      </c>
+      <c r="B16" s="4">
+        <f>B14+B15</f>
+        <v/>
       </c>
       <c r="C16" s="4">
-        <f>B14*(1-B7)</f>
+        <f>C14+C15</f>
         <v/>
       </c>
       <c r="D16" s="4">
-        <f>C16*(1-C7)</f>
+        <f>D14+D15</f>
         <v/>
       </c>
       <c r="E16" s="4">
-        <f>D15</f>
+        <f>D16</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Total Active Umpires</t>
+          <t>Total Games Scored</t>
         </is>
       </c>
       <c r="B17" s="4">
-        <f>B14+B15</f>
+        <f>B16*B10</f>
         <v/>
       </c>
       <c r="C17" s="4">
-        <f>C14+C15</f>
+        <f>C16*C10</f>
         <v/>
       </c>
       <c r="D17" s="4">
-        <f>D14+D15</f>
+        <f>D16*D10</f>
         <v/>
       </c>
       <c r="E17" s="4">
-        <f>D16</f>
+        <f>D17</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Total Games Scored</t>
+          <t>Total Players Reached</t>
         </is>
       </c>
       <c r="B18" s="4">
-        <f>B16*B8</f>
+        <f>B17*B11</f>
         <v/>
       </c>
       <c r="C18" s="4">
-        <f>C16*C8</f>
+        <f>C17*C11</f>
         <v/>
       </c>
       <c r="D18" s="4">
-        <f>D16*D8</f>
+        <f>D17*D11</f>
         <v/>
       </c>
       <c r="E18" s="4">
-        <f>D17</f>
+        <f>D18</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Total Players Reached</t>
+          <t>Total Freemium Users Reached (Parents/Coaches)</t>
         </is>
       </c>
       <c r="B19" s="4">
-        <f>B17*B9</f>
+        <f>B18*B12</f>
         <v/>
       </c>
       <c r="C19" s="4">
-        <f>C17*C9</f>
+        <f>C18*C12</f>
         <v/>
       </c>
       <c r="D19" s="4">
-        <f>D17*D9</f>
+        <f>D18*D12</f>
         <v/>
       </c>
       <c r="E19" s="4">
-        <f>D18</f>
+        <f>D19</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Total Freemium Users Reached (Parents/Coaches)</t>
-        </is>
-      </c>
-      <c r="B20">
-        <f>B18*B10</f>
-        <v/>
-      </c>
-      <c r="C20">
-        <f>C18*C10</f>
-        <v/>
-      </c>
-      <c r="D20">
-        <f>D18*D10</f>
-        <v/>
-      </c>
-      <c r="E20">
-        <f>D19</f>
-        <v/>
-      </c>
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr"/>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
@@ -3779,248 +3763,221 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Year 1</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Year 2</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Year 3</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
+          <t>New Paid Parents</t>
+        </is>
+      </c>
+      <c r="B22" s="4">
+        <f>B19*Assumptions!C8</f>
+        <v/>
+      </c>
+      <c r="C22" s="4">
+        <f>C19*Assumptions!C8</f>
+        <v/>
+      </c>
+      <c r="D22" s="4">
+        <f>D19*Assumptions!C8</f>
+        <v/>
+      </c>
+      <c r="E22" s="4">
+        <f>D22</f>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>New Paid Parents</t>
+          <t>New Paid Coaches</t>
         </is>
       </c>
       <c r="B23" s="4">
-        <f>B19*Assumptions!C8</f>
+        <f>B19*Assumptions!C9</f>
         <v/>
       </c>
       <c r="C23" s="4">
-        <f>C19*Assumptions!C8</f>
+        <f>C19*Assumptions!C9</f>
         <v/>
       </c>
       <c r="D23" s="4">
-        <f>D19*Assumptions!C8</f>
+        <f>D19*Assumptions!C9</f>
         <v/>
       </c>
       <c r="E23" s="4">
-        <f>D22</f>
+        <f>D23</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>New Paid Coaches</t>
-        </is>
-      </c>
-      <c r="B24" s="4">
-        <f>B19*Assumptions!C9</f>
-        <v/>
+          <t>Paid Parents Retained from Prior Year</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="C24" s="4">
-        <f>C19*Assumptions!C9</f>
+        <f>B22*(1-Assumptions!C10)</f>
         <v/>
       </c>
       <c r="D24" s="4">
-        <f>D19*Assumptions!C9</f>
+        <f>C26*(1-Assumptions!C10)</f>
         <v/>
       </c>
       <c r="E24" s="4">
-        <f>D23</f>
+        <f>D24</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Paid Parents Retained from Prior Year</t>
+          <t>Paid Coaches Retained from Prior Year</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C25" s="4">
-        <f>B22*(1-Assumptions!C10)</f>
+        <f>B23*(1-Assumptions!C10)</f>
         <v/>
       </c>
       <c r="D25" s="4">
-        <f>C26*(1-Assumptions!C10)</f>
+        <f>C27*(1-Assumptions!C10)</f>
         <v/>
       </c>
       <c r="E25" s="4">
-        <f>D24</f>
+        <f>D25</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Paid Coaches Retained from Prior Year</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="n">
-        <v>0</v>
+          <t>Total Active Paid Parents</t>
+        </is>
+      </c>
+      <c r="B26" s="4">
+        <f>B22+B24</f>
+        <v/>
       </c>
       <c r="C26" s="4">
-        <f>B23*(1-Assumptions!C10)</f>
+        <f>C22+C24</f>
         <v/>
       </c>
       <c r="D26" s="4">
-        <f>C27*(1-Assumptions!C10)</f>
+        <f>D22+D24</f>
         <v/>
       </c>
       <c r="E26" s="4">
-        <f>D25</f>
+        <f>D26</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Total Active Paid Parents</t>
+          <t>Total Active Paid Coaches</t>
         </is>
       </c>
       <c r="B27" s="4">
-        <f>B22+B24</f>
+        <f>B23+B25</f>
         <v/>
       </c>
       <c r="C27" s="4">
-        <f>C22+C24</f>
+        <f>C23+C25</f>
         <v/>
       </c>
       <c r="D27" s="4">
-        <f>D22+D24</f>
+        <f>D23+D25</f>
         <v/>
       </c>
       <c r="E27" s="4">
-        <f>D26</f>
+        <f>D27</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Total Active Paid Coaches</t>
+          <t>Parent App Revenue</t>
         </is>
       </c>
       <c r="B28" s="6">
-        <f>B23+B25</f>
+        <f>B26*Assumptions!C11</f>
         <v/>
       </c>
       <c r="C28" s="6">
-        <f>C23+C25</f>
+        <f>C26*Assumptions!C11</f>
         <v/>
       </c>
       <c r="D28" s="6">
-        <f>D23+D25</f>
+        <f>D26*Assumptions!C11</f>
         <v/>
       </c>
       <c r="E28" s="6">
-        <f>D27</f>
+        <f>D28</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Parent App Revenue</t>
+          <t>Coach App Revenue</t>
         </is>
       </c>
       <c r="B29" s="6">
-        <f>B26*Assumptions!C11</f>
+        <f>B27*Assumptions!C11</f>
         <v/>
       </c>
       <c r="C29" s="6">
-        <f>C26*Assumptions!C11</f>
+        <f>C27*Assumptions!C11</f>
         <v/>
       </c>
       <c r="D29" s="6">
-        <f>D26*Assumptions!C11</f>
+        <f>D27*Assumptions!C11</f>
         <v/>
       </c>
       <c r="E29" s="6">
-        <f>D28</f>
+        <f>D29</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Coach App Revenue</t>
+          <t>Total ARR</t>
         </is>
       </c>
       <c r="B30" s="6">
-        <f>B27*Assumptions!C11</f>
+        <f>B29+B30</f>
         <v/>
       </c>
       <c r="C30" s="6">
-        <f>C27*Assumptions!C11</f>
+        <f>C29+C30</f>
         <v/>
       </c>
       <c r="D30" s="6">
-        <f>D27*Assumptions!C11</f>
+        <f>D29+D30</f>
         <v/>
       </c>
       <c r="E30" s="6">
-        <f>D29</f>
+        <f>D31</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Total ARR</t>
-        </is>
-      </c>
-      <c r="B31" s="6">
-        <f>B29+B30</f>
-        <v/>
-      </c>
-      <c r="C31" s="6">
-        <f>C29+C30</f>
-        <v/>
-      </c>
+          <t>Total MRR (Avg Year 3)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
       <c r="D31" s="6">
-        <f>D29+D30</f>
-        <v/>
-      </c>
-      <c r="E31" s="6">
-        <f>D31</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Total MRR (Avg Year 3)</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32">
         <f>D31/12</f>
         <v/>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix Cash_Runway #VALUE! errors: Correct Funnel_Model row references for New Paid Parents/Coaches (rows 23-24 instead of 22-23) in Tranche_Detail S&M formulas
</commit_message>
<xml_diff>
--- a/use-of-funds/BLU Use-of-Funds Model.xlsx
+++ b/use-of-funds/BLU Use-of-Funds Model.xlsx
@@ -3007,15 +3007,15 @@
         </is>
       </c>
       <c r="C7" s="6">
-        <f>(Funnel_Model!B22+Funnel_Model!B23)*Assumptions!C17</f>
+        <f>(Funnel_Model!B23+Funnel_Model!B24)*Assumptions!C17</f>
         <v/>
       </c>
       <c r="D7" s="6">
-        <f>(Funnel_Model!C22+Funnel_Model!C23)*Assumptions!C17</f>
+        <f>(Funnel_Model!C23+Funnel_Model!C24)*Assumptions!C17</f>
         <v/>
       </c>
       <c r="E7" s="6">
-        <f>(Funnel_Model!D22+Funnel_Model!D23)*Assumptions!C17</f>
+        <f>(Funnel_Model!D23+Funnel_Model!D24)*Assumptions!C17</f>
         <v/>
       </c>
       <c r="F7" s="6">
@@ -3035,15 +3035,15 @@
         </is>
       </c>
       <c r="C8" s="6">
-        <f>(Funnel_Model!B22+Funnel_Model!B23)*Assumptions!C18</f>
+        <f>(Funnel_Model!B23+Funnel_Model!B24)*Assumptions!C18</f>
         <v/>
       </c>
       <c r="D8" s="6">
-        <f>(Funnel_Model!C22+Funnel_Model!C23)*Assumptions!C18</f>
+        <f>(Funnel_Model!C23+Funnel_Model!C24)*Assumptions!C18</f>
         <v/>
       </c>
       <c r="E8" s="6">
-        <f>(Funnel_Model!D22+Funnel_Model!D23)*Assumptions!C18</f>
+        <f>(Funnel_Model!D23+Funnel_Model!D24)*Assumptions!C18</f>
         <v/>
       </c>
       <c r="F8" s="6">

</xml_diff>